<commit_message>
Gem mine valg (sport + danske backdrops) 2026-10-05 16:09:55
</commit_message>
<xml_diff>
--- a/data/sport_artwork_review.xlsx
+++ b/data/sport_artwork_review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EPGoal\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90078082-294F-429F-BDE3-7C2FC4459CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{991F2DD8-260F-4E3D-A73B-7D405737BC50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2936" uniqueCount="810">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2936" uniqueCount="811">
   <si>
     <t>Kanalgruppe</t>
   </si>
@@ -2457,6 +2457,9 @@
   </si>
   <si>
     <t>Rækker der ikke længere er aktuelle, men SOM havde et udfyldt valg (og ikke er ignoreret), havner i arket 'Forsvundne (havde valg)' - intet forsvinder usporligt.</t>
+  </si>
+  <si>
+    <t>TMDB</t>
   </si>
 </sst>
 </file>
@@ -5913,9 +5916,9 @@
         <v>418</v>
       </c>
       <c r="D181" t="s">
-        <v>419</v>
-      </c>
-      <c r="G181" t="s">
+        <v>810</v>
+      </c>
+      <c r="F181" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9120,15 +9123,15 @@
         <v>8</v>
       </c>
       <c r="B370" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C370" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D370" t="s">
-        <v>23</v>
-      </c>
-      <c r="F370" t="s">
+        <v>11</v>
+      </c>
+      <c r="G370" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9137,15 +9140,15 @@
         <v>8</v>
       </c>
       <c r="B371" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="C371" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="D371" t="s">
-        <v>25</v>
-      </c>
-      <c r="F371" t="s">
+        <v>11</v>
+      </c>
+      <c r="G371" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9154,15 +9157,15 @@
         <v>8</v>
       </c>
       <c r="B372" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C372" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="D372" t="s">
-        <v>28</v>
-      </c>
-      <c r="F372" t="s">
+        <v>11</v>
+      </c>
+      <c r="G372" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9171,18 +9174,15 @@
         <v>8</v>
       </c>
       <c r="B373" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C373" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="D373" t="s">
-        <v>31</v>
-      </c>
-      <c r="E373" t="s">
-        <v>31</v>
-      </c>
-      <c r="F373" t="s">
+        <v>11</v>
+      </c>
+      <c r="G373" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9191,18 +9191,15 @@
         <v>8</v>
       </c>
       <c r="B374" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C374" t="s">
-        <v>32</v>
+        <v>82</v>
       </c>
       <c r="D374" t="s">
-        <v>33</v>
-      </c>
-      <c r="E374" t="s">
-        <v>33</v>
-      </c>
-      <c r="F374" t="s">
+        <v>11</v>
+      </c>
+      <c r="G374" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9211,18 +9208,15 @@
         <v>8</v>
       </c>
       <c r="B375" t="s">
-        <v>35</v>
+        <v>88</v>
       </c>
       <c r="C375" t="s">
-        <v>36</v>
+        <v>89</v>
       </c>
       <c r="D375" t="s">
-        <v>37</v>
-      </c>
-      <c r="E375" t="s">
-        <v>37</v>
-      </c>
-      <c r="F375" t="s">
+        <v>11</v>
+      </c>
+      <c r="G375" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9231,18 +9225,15 @@
         <v>8</v>
       </c>
       <c r="B376" t="s">
-        <v>38</v>
+        <v>88</v>
       </c>
       <c r="C376" t="s">
-        <v>39</v>
+        <v>97</v>
       </c>
       <c r="D376" t="s">
-        <v>37</v>
-      </c>
-      <c r="E376" t="s">
-        <v>37</v>
-      </c>
-      <c r="F376" t="s">
+        <v>11</v>
+      </c>
+      <c r="G376" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9251,18 +9242,15 @@
         <v>8</v>
       </c>
       <c r="B377" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="C377" t="s">
-        <v>45</v>
+        <v>101</v>
       </c>
       <c r="D377" t="s">
-        <v>37</v>
-      </c>
-      <c r="E377" t="s">
-        <v>37</v>
-      </c>
-      <c r="F377" t="s">
+        <v>11</v>
+      </c>
+      <c r="G377" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9271,18 +9259,15 @@
         <v>8</v>
       </c>
       <c r="B378" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="C378" t="s">
-        <v>46</v>
+        <v>106</v>
       </c>
       <c r="D378" t="s">
-        <v>37</v>
-      </c>
-      <c r="E378" t="s">
-        <v>37</v>
-      </c>
-      <c r="F378" t="s">
+        <v>11</v>
+      </c>
+      <c r="G378" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9291,18 +9276,15 @@
         <v>8</v>
       </c>
       <c r="B379" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="C379" t="s">
-        <v>48</v>
+        <v>114</v>
       </c>
       <c r="D379" t="s">
-        <v>37</v>
-      </c>
-      <c r="E379" t="s">
-        <v>37</v>
-      </c>
-      <c r="F379" t="s">
+        <v>11</v>
+      </c>
+      <c r="G379" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9311,18 +9293,15 @@
         <v>8</v>
       </c>
       <c r="B380" t="s">
-        <v>26</v>
+        <v>88</v>
       </c>
       <c r="C380" t="s">
-        <v>49</v>
+        <v>126</v>
       </c>
       <c r="D380" t="s">
-        <v>37</v>
-      </c>
-      <c r="E380" t="s">
-        <v>37</v>
-      </c>
-      <c r="F380" t="s">
+        <v>11</v>
+      </c>
+      <c r="G380" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9331,18 +9310,15 @@
         <v>8</v>
       </c>
       <c r="B381" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="C381" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
       <c r="D381" t="s">
-        <v>37</v>
-      </c>
-      <c r="E381" t="s">
-        <v>37</v>
-      </c>
-      <c r="F381" t="s">
+        <v>11</v>
+      </c>
+      <c r="G381" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9351,18 +9327,15 @@
         <v>8</v>
       </c>
       <c r="B382" t="s">
-        <v>26</v>
+        <v>88</v>
       </c>
       <c r="C382" t="s">
-        <v>51</v>
+        <v>133</v>
       </c>
       <c r="D382" t="s">
-        <v>52</v>
-      </c>
-      <c r="E382" t="s">
-        <v>52</v>
-      </c>
-      <c r="F382" t="s">
+        <v>11</v>
+      </c>
+      <c r="G382" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9371,15 +9344,15 @@
         <v>8</v>
       </c>
       <c r="B383" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="C383" t="s">
-        <v>55</v>
+        <v>141</v>
       </c>
       <c r="D383" t="s">
-        <v>56</v>
-      </c>
-      <c r="F383" t="s">
+        <v>11</v>
+      </c>
+      <c r="G383" t="s">
         <v>12</v>
       </c>
     </row>
@@ -9388,611 +9361,581 @@
         <v>8</v>
       </c>
       <c r="B384" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="C384" t="s">
-        <v>63</v>
+        <v>146</v>
       </c>
       <c r="D384" t="s">
-        <v>52</v>
-      </c>
-      <c r="F384" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="385" spans="1:6" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="G384" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="385" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
         <v>8</v>
       </c>
       <c r="B385" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="C385" t="s">
-        <v>65</v>
+        <v>158</v>
       </c>
       <c r="D385" t="s">
+        <v>11</v>
+      </c>
+      <c r="G385" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="386" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A386" t="s">
+        <v>8</v>
+      </c>
+      <c r="B386" t="s">
+        <v>17</v>
+      </c>
+      <c r="C386" t="s">
+        <v>177</v>
+      </c>
+      <c r="D386" t="s">
+        <v>11</v>
+      </c>
+      <c r="G386" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="387" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A387" t="s">
+        <v>179</v>
+      </c>
+      <c r="B387" t="s">
+        <v>182</v>
+      </c>
+      <c r="C387" t="s">
+        <v>186</v>
+      </c>
+      <c r="D387" t="s">
+        <v>11</v>
+      </c>
+      <c r="G387" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="388" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A388" t="s">
+        <v>179</v>
+      </c>
+      <c r="B388" t="s">
+        <v>182</v>
+      </c>
+      <c r="C388" t="s">
+        <v>189</v>
+      </c>
+      <c r="D388" t="s">
+        <v>11</v>
+      </c>
+      <c r="G388" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="389" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A389" t="s">
+        <v>179</v>
+      </c>
+      <c r="B389" t="s">
+        <v>182</v>
+      </c>
+      <c r="C389" t="s">
+        <v>192</v>
+      </c>
+      <c r="D389" t="s">
+        <v>11</v>
+      </c>
+      <c r="G389" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="390" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A390" t="s">
+        <v>179</v>
+      </c>
+      <c r="B390" t="s">
+        <v>182</v>
+      </c>
+      <c r="C390" t="s">
+        <v>196</v>
+      </c>
+      <c r="D390" t="s">
+        <v>11</v>
+      </c>
+      <c r="G390" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="391" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A391" t="s">
+        <v>179</v>
+      </c>
+      <c r="B391" t="s">
+        <v>182</v>
+      </c>
+      <c r="C391" t="s">
+        <v>197</v>
+      </c>
+      <c r="D391" t="s">
+        <v>11</v>
+      </c>
+      <c r="G391" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="392" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A392" t="s">
+        <v>179</v>
+      </c>
+      <c r="B392" t="s">
+        <v>203</v>
+      </c>
+      <c r="C392" t="s">
+        <v>215</v>
+      </c>
+      <c r="D392" t="s">
+        <v>11</v>
+      </c>
+      <c r="G392" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="393" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A393" t="s">
+        <v>179</v>
+      </c>
+      <c r="B393" t="s">
+        <v>203</v>
+      </c>
+      <c r="C393" t="s">
+        <v>242</v>
+      </c>
+      <c r="D393" t="s">
+        <v>11</v>
+      </c>
+      <c r="G393" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="394" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A394" t="s">
+        <v>179</v>
+      </c>
+      <c r="B394" t="s">
+        <v>182</v>
+      </c>
+      <c r="C394" t="s">
+        <v>246</v>
+      </c>
+      <c r="D394" t="s">
+        <v>11</v>
+      </c>
+      <c r="G394" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="395" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A395" t="s">
+        <v>179</v>
+      </c>
+      <c r="B395" t="s">
+        <v>182</v>
+      </c>
+      <c r="C395" t="s">
+        <v>247</v>
+      </c>
+      <c r="D395" t="s">
+        <v>11</v>
+      </c>
+      <c r="G395" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="396" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A396" t="s">
+        <v>179</v>
+      </c>
+      <c r="B396" t="s">
+        <v>182</v>
+      </c>
+      <c r="C396" t="s">
+        <v>250</v>
+      </c>
+      <c r="D396" t="s">
+        <v>11</v>
+      </c>
+      <c r="G396" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="397" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A397" t="s">
+        <v>179</v>
+      </c>
+      <c r="B397" t="s">
+        <v>180</v>
+      </c>
+      <c r="C397" t="s">
+        <v>252</v>
+      </c>
+      <c r="D397" t="s">
+        <v>11</v>
+      </c>
+      <c r="G397" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="398" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A398" t="s">
+        <v>179</v>
+      </c>
+      <c r="B398" t="s">
+        <v>182</v>
+      </c>
+      <c r="C398" t="s">
+        <v>253</v>
+      </c>
+      <c r="D398" t="s">
+        <v>11</v>
+      </c>
+      <c r="G398" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="399" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A399" t="s">
+        <v>179</v>
+      </c>
+      <c r="B399" t="s">
+        <v>182</v>
+      </c>
+      <c r="C399" t="s">
+        <v>255</v>
+      </c>
+      <c r="D399" t="s">
+        <v>11</v>
+      </c>
+      <c r="G399" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="400" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A400" t="s">
+        <v>179</v>
+      </c>
+      <c r="B400" t="s">
+        <v>182</v>
+      </c>
+      <c r="C400" t="s">
+        <v>276</v>
+      </c>
+      <c r="D400" t="s">
+        <v>11</v>
+      </c>
+      <c r="G400" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="401" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A401" t="s">
+        <v>179</v>
+      </c>
+      <c r="B401" t="s">
+        <v>182</v>
+      </c>
+      <c r="C401" t="s">
+        <v>279</v>
+      </c>
+      <c r="D401" t="s">
+        <v>11</v>
+      </c>
+      <c r="G401" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="402" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A402" t="s">
+        <v>179</v>
+      </c>
+      <c r="B402" t="s">
+        <v>203</v>
+      </c>
+      <c r="C402" t="s">
+        <v>280</v>
+      </c>
+      <c r="D402" t="s">
+        <v>11</v>
+      </c>
+      <c r="G402" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="403" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A403" t="s">
+        <v>179</v>
+      </c>
+      <c r="B403" t="s">
+        <v>203</v>
+      </c>
+      <c r="C403" t="s">
+        <v>282</v>
+      </c>
+      <c r="D403" t="s">
+        <v>11</v>
+      </c>
+      <c r="G403" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="404" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A404" t="s">
+        <v>179</v>
+      </c>
+      <c r="B404" t="s">
+        <v>264</v>
+      </c>
+      <c r="C404" t="s">
+        <v>286</v>
+      </c>
+      <c r="D404" t="s">
+        <v>207</v>
+      </c>
+      <c r="G404" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="405" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A405" t="s">
+        <v>179</v>
+      </c>
+      <c r="B405" t="s">
+        <v>264</v>
+      </c>
+      <c r="C405" t="s">
+        <v>290</v>
+      </c>
+      <c r="D405" t="s">
+        <v>268</v>
+      </c>
+      <c r="G405" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="406" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A406" t="s">
+        <v>8</v>
+      </c>
+      <c r="B406" t="s">
+        <v>21</v>
+      </c>
+      <c r="C406" t="s">
+        <v>22</v>
+      </c>
+      <c r="D406" t="s">
+        <v>23</v>
+      </c>
+      <c r="F406" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="407" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A407" t="s">
+        <v>8</v>
+      </c>
+      <c r="B407" t="s">
+        <v>21</v>
+      </c>
+      <c r="C407" t="s">
+        <v>24</v>
+      </c>
+      <c r="D407" t="s">
+        <v>25</v>
+      </c>
+      <c r="F407" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="408" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A408" t="s">
+        <v>8</v>
+      </c>
+      <c r="B408" t="s">
+        <v>26</v>
+      </c>
+      <c r="C408" t="s">
+        <v>27</v>
+      </c>
+      <c r="D408" t="s">
         <v>28</v>
       </c>
-      <c r="F385" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="386" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A386" t="s">
-        <v>8</v>
-      </c>
-      <c r="B386" t="s">
+      <c r="F408" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="409" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A409" t="s">
+        <v>8</v>
+      </c>
+      <c r="B409" t="s">
+        <v>29</v>
+      </c>
+      <c r="C409" t="s">
+        <v>30</v>
+      </c>
+      <c r="D409" t="s">
+        <v>31</v>
+      </c>
+      <c r="E409" t="s">
+        <v>31</v>
+      </c>
+      <c r="F409" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="410" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A410" t="s">
+        <v>8</v>
+      </c>
+      <c r="B410" t="s">
+        <v>26</v>
+      </c>
+      <c r="C410" t="s">
+        <v>32</v>
+      </c>
+      <c r="D410" t="s">
+        <v>33</v>
+      </c>
+      <c r="E410" t="s">
+        <v>33</v>
+      </c>
+      <c r="F410" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="411" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A411" t="s">
+        <v>8</v>
+      </c>
+      <c r="B411" t="s">
+        <v>35</v>
+      </c>
+      <c r="C411" t="s">
+        <v>36</v>
+      </c>
+      <c r="D411" t="s">
+        <v>37</v>
+      </c>
+      <c r="E411" t="s">
+        <v>37</v>
+      </c>
+      <c r="F411" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="412" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A412" t="s">
+        <v>8</v>
+      </c>
+      <c r="B412" t="s">
         <v>38</v>
       </c>
-      <c r="C386" t="s">
-        <v>69</v>
-      </c>
-      <c r="D386" t="s">
-        <v>52</v>
-      </c>
-      <c r="E386" t="s">
-        <v>52</v>
-      </c>
-      <c r="F386" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="387" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A387" t="s">
-        <v>8</v>
-      </c>
-      <c r="B387" t="s">
-        <v>15</v>
-      </c>
-      <c r="C387" t="s">
-        <v>70</v>
-      </c>
-      <c r="D387" t="s">
-        <v>52</v>
-      </c>
-      <c r="E387" t="s">
-        <v>52</v>
-      </c>
-      <c r="F387" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="388" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A388" t="s">
-        <v>8</v>
-      </c>
-      <c r="B388" t="s">
-        <v>21</v>
-      </c>
-      <c r="C388" t="s">
-        <v>78</v>
-      </c>
-      <c r="D388" t="s">
-        <v>11</v>
-      </c>
-      <c r="F388" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="389" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A389" t="s">
-        <v>8</v>
-      </c>
-      <c r="B389" t="s">
-        <v>54</v>
-      </c>
-      <c r="C389" t="s">
-        <v>84</v>
-      </c>
-      <c r="D389" t="s">
-        <v>85</v>
-      </c>
-      <c r="F389" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="390" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A390" t="s">
-        <v>8</v>
-      </c>
-      <c r="B390" t="s">
+      <c r="C412" t="s">
+        <v>39</v>
+      </c>
+      <c r="D412" t="s">
+        <v>37</v>
+      </c>
+      <c r="E412" t="s">
+        <v>37</v>
+      </c>
+      <c r="F412" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="413" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A413" t="s">
+        <v>8</v>
+      </c>
+      <c r="B413" t="s">
+        <v>44</v>
+      </c>
+      <c r="C413" t="s">
+        <v>45</v>
+      </c>
+      <c r="D413" t="s">
+        <v>37</v>
+      </c>
+      <c r="E413" t="s">
+        <v>37</v>
+      </c>
+      <c r="F413" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="414" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A414" t="s">
+        <v>8</v>
+      </c>
+      <c r="B414" t="s">
         <v>26</v>
       </c>
-      <c r="C390" t="s">
-        <v>94</v>
-      </c>
-      <c r="D390" t="s">
-        <v>95</v>
-      </c>
-      <c r="F390" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="391" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A391" t="s">
-        <v>8</v>
-      </c>
-      <c r="B391" t="s">
-        <v>35</v>
-      </c>
-      <c r="C391" t="s">
-        <v>109</v>
-      </c>
-      <c r="D391" t="s">
-        <v>105</v>
-      </c>
-      <c r="E391" t="s">
-        <v>105</v>
-      </c>
-      <c r="F391" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="392" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A392" t="s">
-        <v>8</v>
-      </c>
-      <c r="B392" t="s">
-        <v>38</v>
-      </c>
-      <c r="C392" t="s">
-        <v>110</v>
-      </c>
-      <c r="D392" t="s">
-        <v>105</v>
-      </c>
-      <c r="E392" t="s">
-        <v>105</v>
-      </c>
-      <c r="F392" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="393" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A393" t="s">
-        <v>8</v>
-      </c>
-      <c r="B393" t="s">
+      <c r="C414" t="s">
+        <v>46</v>
+      </c>
+      <c r="D414" t="s">
+        <v>37</v>
+      </c>
+      <c r="E414" t="s">
+        <v>37</v>
+      </c>
+      <c r="F414" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="415" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A415" t="s">
+        <v>8</v>
+      </c>
+      <c r="B415" t="s">
+        <v>47</v>
+      </c>
+      <c r="C415" t="s">
+        <v>48</v>
+      </c>
+      <c r="D415" t="s">
+        <v>37</v>
+      </c>
+      <c r="E415" t="s">
+        <v>37</v>
+      </c>
+      <c r="F415" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="416" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A416" t="s">
+        <v>8</v>
+      </c>
+      <c r="B416" t="s">
         <v>26</v>
       </c>
-      <c r="C393" t="s">
-        <v>111</v>
-      </c>
-      <c r="D393" t="s">
-        <v>105</v>
-      </c>
-      <c r="E393" t="s">
-        <v>105</v>
-      </c>
-      <c r="F393" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="394" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A394" t="s">
-        <v>8</v>
-      </c>
-      <c r="B394" t="s">
-        <v>38</v>
-      </c>
-      <c r="C394" t="s">
-        <v>112</v>
-      </c>
-      <c r="D394" t="s">
-        <v>105</v>
-      </c>
-      <c r="E394" t="s">
-        <v>105</v>
-      </c>
-      <c r="F394" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="395" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A395" t="s">
-        <v>8</v>
-      </c>
-      <c r="B395" t="s">
-        <v>21</v>
-      </c>
-      <c r="C395" t="s">
-        <v>121</v>
-      </c>
-      <c r="D395" t="s">
-        <v>122</v>
-      </c>
-      <c r="F395" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="396" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A396" t="s">
-        <v>8</v>
-      </c>
-      <c r="B396" t="s">
-        <v>147</v>
-      </c>
-      <c r="C396" t="s">
-        <v>148</v>
-      </c>
-      <c r="D396" t="s">
-        <v>149</v>
-      </c>
-      <c r="F396" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="397" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A397" t="s">
-        <v>8</v>
-      </c>
-      <c r="B397" t="s">
-        <v>147</v>
-      </c>
-      <c r="C397" t="s">
-        <v>150</v>
-      </c>
-      <c r="D397" t="s">
-        <v>149</v>
-      </c>
-      <c r="F397" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="398" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A398" t="s">
-        <v>8</v>
-      </c>
-      <c r="B398" t="s">
-        <v>147</v>
-      </c>
-      <c r="C398" t="s">
-        <v>151</v>
-      </c>
-      <c r="D398" t="s">
-        <v>152</v>
-      </c>
-      <c r="F398" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="399" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A399" t="s">
-        <v>8</v>
-      </c>
-      <c r="B399" t="s">
-        <v>153</v>
-      </c>
-      <c r="C399" t="s">
-        <v>154</v>
-      </c>
-      <c r="D399" t="s">
-        <v>155</v>
-      </c>
-      <c r="F399" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="400" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A400" t="s">
-        <v>8</v>
-      </c>
-      <c r="B400" t="s">
-        <v>147</v>
-      </c>
-      <c r="C400" t="s">
-        <v>156</v>
-      </c>
-      <c r="D400" t="s">
-        <v>155</v>
-      </c>
-      <c r="E400" t="s">
-        <v>155</v>
-      </c>
-      <c r="F400" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="401" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A401" t="s">
-        <v>8</v>
-      </c>
-      <c r="B401" t="s">
-        <v>135</v>
-      </c>
-      <c r="C401" t="s">
-        <v>163</v>
-      </c>
-      <c r="D401" t="s">
-        <v>164</v>
-      </c>
-      <c r="F401" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="402" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A402" t="s">
-        <v>8</v>
-      </c>
-      <c r="B402" t="s">
-        <v>166</v>
-      </c>
-      <c r="C402" t="s">
-        <v>167</v>
-      </c>
-      <c r="D402" t="s">
-        <v>168</v>
-      </c>
-      <c r="E402" t="s">
-        <v>168</v>
-      </c>
-      <c r="F402" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="403" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A403" t="s">
-        <v>8</v>
-      </c>
-      <c r="B403" t="s">
-        <v>169</v>
-      </c>
-      <c r="C403" t="s">
-        <v>170</v>
-      </c>
-      <c r="D403" t="s">
-        <v>168</v>
-      </c>
-      <c r="E403" t="s">
-        <v>168</v>
-      </c>
-      <c r="F403" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="404" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A404" t="s">
-        <v>8</v>
-      </c>
-      <c r="B404" t="s">
-        <v>15</v>
-      </c>
-      <c r="C404" t="s">
-        <v>172</v>
-      </c>
-      <c r="D404" t="s">
-        <v>11</v>
-      </c>
-      <c r="F404" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="405" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A405" t="s">
-        <v>8</v>
-      </c>
-      <c r="B405" t="s">
-        <v>147</v>
-      </c>
-      <c r="C405" t="s">
-        <v>173</v>
-      </c>
-      <c r="D405" t="s">
-        <v>174</v>
-      </c>
-      <c r="E405" t="s">
-        <v>174</v>
-      </c>
-      <c r="F405" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="406" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A406" t="s">
-        <v>179</v>
-      </c>
-      <c r="B406" t="s">
-        <v>198</v>
-      </c>
-      <c r="C406" t="s">
-        <v>199</v>
-      </c>
-      <c r="D406" t="s">
-        <v>200</v>
-      </c>
-      <c r="F406" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="407" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A407" t="s">
-        <v>179</v>
-      </c>
-      <c r="B407" t="s">
-        <v>198</v>
-      </c>
-      <c r="C407" t="s">
-        <v>201</v>
-      </c>
-      <c r="D407" t="s">
-        <v>200</v>
-      </c>
-      <c r="F407" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="408" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A408" t="s">
-        <v>179</v>
-      </c>
-      <c r="B408" t="s">
-        <v>198</v>
-      </c>
-      <c r="C408" t="s">
-        <v>202</v>
-      </c>
-      <c r="D408" t="s">
-        <v>200</v>
-      </c>
-      <c r="F408" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="409" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A409" t="s">
-        <v>179</v>
-      </c>
-      <c r="B409" t="s">
-        <v>218</v>
-      </c>
-      <c r="C409" t="s">
-        <v>219</v>
-      </c>
-      <c r="D409" t="s">
-        <v>220</v>
-      </c>
-      <c r="E409" t="s">
-        <v>220</v>
-      </c>
-      <c r="F409" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="410" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A410" t="s">
-        <v>179</v>
-      </c>
-      <c r="B410" t="s">
-        <v>221</v>
-      </c>
-      <c r="C410" t="s">
-        <v>222</v>
-      </c>
-      <c r="D410" t="s">
-        <v>220</v>
-      </c>
-      <c r="E410" t="s">
-        <v>220</v>
-      </c>
-      <c r="F410" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="411" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A411" t="s">
-        <v>179</v>
-      </c>
-      <c r="B411" t="s">
-        <v>223</v>
-      </c>
-      <c r="C411" t="s">
-        <v>224</v>
-      </c>
-      <c r="D411" t="s">
-        <v>220</v>
-      </c>
-      <c r="E411" t="s">
-        <v>220</v>
-      </c>
-      <c r="F411" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="412" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A412" t="s">
-        <v>179</v>
-      </c>
-      <c r="B412" t="s">
-        <v>225</v>
-      </c>
-      <c r="C412" t="s">
-        <v>226</v>
-      </c>
-      <c r="D412" t="s">
-        <v>220</v>
-      </c>
-      <c r="E412" t="s">
-        <v>220</v>
-      </c>
-      <c r="F412" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="413" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A413" t="s">
-        <v>179</v>
-      </c>
-      <c r="B413" t="s">
-        <v>225</v>
-      </c>
-      <c r="C413" t="s">
-        <v>227</v>
-      </c>
-      <c r="D413" t="s">
-        <v>220</v>
-      </c>
-      <c r="E413" t="s">
-        <v>220</v>
-      </c>
-      <c r="F413" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="414" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A414" t="s">
-        <v>179</v>
-      </c>
-      <c r="B414" t="s">
-        <v>225</v>
-      </c>
-      <c r="C414" t="s">
-        <v>228</v>
-      </c>
-      <c r="D414" t="s">
-        <v>220</v>
-      </c>
-      <c r="E414" t="s">
-        <v>220</v>
-      </c>
-      <c r="F414" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="415" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A415" t="s">
-        <v>179</v>
-      </c>
-      <c r="B415" t="s">
-        <v>225</v>
-      </c>
-      <c r="C415" t="s">
-        <v>229</v>
-      </c>
-      <c r="D415" t="s">
-        <v>220</v>
-      </c>
-      <c r="E415" t="s">
-        <v>220</v>
-      </c>
-      <c r="F415" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="416" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A416" t="s">
-        <v>179</v>
-      </c>
-      <c r="B416" t="s">
-        <v>225</v>
-      </c>
       <c r="C416" t="s">
-        <v>231</v>
+        <v>49</v>
       </c>
       <c r="D416" t="s">
-        <v>220</v>
+        <v>37</v>
       </c>
       <c r="E416" t="s">
-        <v>220</v>
+        <v>37</v>
       </c>
       <c r="F416" t="s">
         <v>12</v>
@@ -10000,19 +9943,19 @@
     </row>
     <row r="417" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B417" t="s">
-        <v>225</v>
+        <v>47</v>
       </c>
       <c r="C417" t="s">
-        <v>232</v>
+        <v>50</v>
       </c>
       <c r="D417" t="s">
-        <v>220</v>
+        <v>37</v>
       </c>
       <c r="E417" t="s">
-        <v>220</v>
+        <v>37</v>
       </c>
       <c r="F417" t="s">
         <v>12</v>
@@ -10020,19 +9963,19 @@
     </row>
     <row r="418" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B418" t="s">
-        <v>225</v>
+        <v>26</v>
       </c>
       <c r="C418" t="s">
-        <v>233</v>
+        <v>51</v>
       </c>
       <c r="D418" t="s">
-        <v>220</v>
+        <v>52</v>
       </c>
       <c r="E418" t="s">
-        <v>220</v>
+        <v>52</v>
       </c>
       <c r="F418" t="s">
         <v>12</v>
@@ -10040,19 +9983,16 @@
     </row>
     <row r="419" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B419" t="s">
-        <v>234</v>
+        <v>54</v>
       </c>
       <c r="C419" t="s">
-        <v>235</v>
+        <v>55</v>
       </c>
       <c r="D419" t="s">
-        <v>220</v>
-      </c>
-      <c r="E419" t="s">
-        <v>220</v>
+        <v>56</v>
       </c>
       <c r="F419" t="s">
         <v>12</v>
@@ -10060,19 +10000,16 @@
     </row>
     <row r="420" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B420" t="s">
-        <v>225</v>
+        <v>62</v>
       </c>
       <c r="C420" t="s">
-        <v>237</v>
+        <v>63</v>
       </c>
       <c r="D420" t="s">
-        <v>220</v>
-      </c>
-      <c r="E420" t="s">
-        <v>220</v>
+        <v>52</v>
       </c>
       <c r="F420" t="s">
         <v>12</v>
@@ -10080,19 +10017,16 @@
     </row>
     <row r="421" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B421" t="s">
-        <v>225</v>
+        <v>64</v>
       </c>
       <c r="C421" t="s">
-        <v>239</v>
+        <v>65</v>
       </c>
       <c r="D421" t="s">
-        <v>220</v>
-      </c>
-      <c r="E421" t="s">
-        <v>220</v>
+        <v>28</v>
       </c>
       <c r="F421" t="s">
         <v>12</v>
@@ -10100,19 +10034,19 @@
     </row>
     <row r="422" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B422" t="s">
-        <v>225</v>
+        <v>38</v>
       </c>
       <c r="C422" t="s">
-        <v>240</v>
+        <v>69</v>
       </c>
       <c r="D422" t="s">
-        <v>220</v>
+        <v>52</v>
       </c>
       <c r="E422" t="s">
-        <v>220</v>
+        <v>52</v>
       </c>
       <c r="F422" t="s">
         <v>12</v>
@@ -10120,16 +10054,19 @@
     </row>
     <row r="423" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B423" t="s">
-        <v>198</v>
+        <v>15</v>
       </c>
       <c r="C423" t="s">
-        <v>256</v>
+        <v>70</v>
       </c>
       <c r="D423" t="s">
-        <v>28</v>
+        <v>52</v>
+      </c>
+      <c r="E423" t="s">
+        <v>52</v>
       </c>
       <c r="F423" t="s">
         <v>12</v>
@@ -10137,19 +10074,16 @@
     </row>
     <row r="424" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B424" t="s">
-        <v>198</v>
+        <v>21</v>
       </c>
       <c r="C424" t="s">
-        <v>258</v>
+        <v>78</v>
       </c>
       <c r="D424" t="s">
-        <v>259</v>
-      </c>
-      <c r="E424" t="s">
-        <v>259</v>
+        <v>11</v>
       </c>
       <c r="F424" t="s">
         <v>12</v>
@@ -10157,16 +10091,16 @@
     </row>
     <row r="425" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B425" t="s">
-        <v>262</v>
+        <v>54</v>
       </c>
       <c r="C425" t="s">
-        <v>263</v>
+        <v>84</v>
       </c>
       <c r="D425" t="s">
-        <v>259</v>
+        <v>85</v>
       </c>
       <c r="F425" t="s">
         <v>12</v>
@@ -10174,16 +10108,16 @@
     </row>
     <row r="426" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B426" t="s">
-        <v>264</v>
+        <v>26</v>
       </c>
       <c r="C426" t="s">
-        <v>265</v>
+        <v>94</v>
       </c>
       <c r="D426" t="s">
-        <v>259</v>
+        <v>95</v>
       </c>
       <c r="F426" t="s">
         <v>12</v>
@@ -10191,16 +10125,19 @@
     </row>
     <row r="427" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B427" t="s">
-        <v>205</v>
+        <v>35</v>
       </c>
       <c r="C427" t="s">
-        <v>266</v>
+        <v>109</v>
       </c>
       <c r="D427" t="s">
-        <v>259</v>
+        <v>105</v>
+      </c>
+      <c r="E427" t="s">
+        <v>105</v>
       </c>
       <c r="F427" t="s">
         <v>12</v>
@@ -10208,16 +10145,19 @@
     </row>
     <row r="428" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B428" t="s">
-        <v>264</v>
+        <v>38</v>
       </c>
       <c r="C428" t="s">
-        <v>267</v>
+        <v>110</v>
       </c>
       <c r="D428" t="s">
-        <v>268</v>
+        <v>105</v>
+      </c>
+      <c r="E428" t="s">
+        <v>105</v>
       </c>
       <c r="F428" t="s">
         <v>12</v>
@@ -10225,16 +10165,19 @@
     </row>
     <row r="429" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B429" t="s">
-        <v>205</v>
+        <v>26</v>
       </c>
       <c r="C429" t="s">
-        <v>269</v>
+        <v>111</v>
       </c>
       <c r="D429" t="s">
-        <v>259</v>
+        <v>105</v>
+      </c>
+      <c r="E429" t="s">
+        <v>105</v>
       </c>
       <c r="F429" t="s">
         <v>12</v>
@@ -10242,19 +10185,19 @@
     </row>
     <row r="430" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B430" t="s">
-        <v>205</v>
+        <v>38</v>
       </c>
       <c r="C430" t="s">
-        <v>270</v>
+        <v>112</v>
       </c>
       <c r="D430" t="s">
-        <v>271</v>
+        <v>105</v>
       </c>
       <c r="E430" t="s">
-        <v>271</v>
+        <v>105</v>
       </c>
       <c r="F430" t="s">
         <v>12</v>
@@ -10262,19 +10205,16 @@
     </row>
     <row r="431" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B431" t="s">
-        <v>262</v>
+        <v>21</v>
       </c>
       <c r="C431" t="s">
-        <v>285</v>
+        <v>121</v>
       </c>
       <c r="D431" t="s">
-        <v>268</v>
-      </c>
-      <c r="E431" t="s">
-        <v>268</v>
+        <v>122</v>
       </c>
       <c r="F431" t="s">
         <v>12</v>
@@ -10282,205 +10222,184 @@
     </row>
     <row r="432" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B432" t="s">
-        <v>264</v>
+        <v>147</v>
       </c>
       <c r="C432" t="s">
-        <v>287</v>
+        <v>148</v>
       </c>
       <c r="D432" t="s">
-        <v>288</v>
-      </c>
-      <c r="E432" t="s">
-        <v>288</v>
+        <v>149</v>
       </c>
       <c r="F432" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="433" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B433" t="s">
-        <v>262</v>
+        <v>147</v>
       </c>
       <c r="C433" t="s">
-        <v>289</v>
+        <v>150</v>
       </c>
       <c r="D433" t="s">
-        <v>268</v>
-      </c>
-      <c r="E433" t="s">
-        <v>268</v>
+        <v>149</v>
       </c>
       <c r="F433" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="434" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B434" t="s">
-        <v>264</v>
+        <v>147</v>
       </c>
       <c r="C434" t="s">
-        <v>291</v>
+        <v>151</v>
       </c>
       <c r="D434" t="s">
-        <v>288</v>
-      </c>
-      <c r="E434" t="s">
-        <v>288</v>
+        <v>152</v>
       </c>
       <c r="F434" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="435" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B435" t="s">
-        <v>262</v>
+        <v>153</v>
       </c>
       <c r="C435" t="s">
-        <v>292</v>
+        <v>154</v>
       </c>
       <c r="D435" t="s">
-        <v>293</v>
-      </c>
-      <c r="E435" t="s">
-        <v>293</v>
+        <v>155</v>
       </c>
       <c r="F435" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="436" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B436" t="s">
-        <v>264</v>
+        <v>147</v>
       </c>
       <c r="C436" t="s">
-        <v>294</v>
+        <v>156</v>
       </c>
       <c r="D436" t="s">
-        <v>293</v>
+        <v>155</v>
       </c>
       <c r="E436" t="s">
-        <v>293</v>
+        <v>155</v>
       </c>
       <c r="F436" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="437" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B437" t="s">
-        <v>198</v>
+        <v>135</v>
       </c>
       <c r="C437" t="s">
-        <v>296</v>
+        <v>163</v>
       </c>
       <c r="D437" t="s">
-        <v>220</v>
-      </c>
-      <c r="E437" t="s">
-        <v>220</v>
+        <v>164</v>
       </c>
       <c r="F437" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="438" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B438" t="s">
-        <v>198</v>
+        <v>166</v>
       </c>
       <c r="C438" t="s">
-        <v>302</v>
+        <v>167</v>
       </c>
       <c r="D438" t="s">
-        <v>220</v>
+        <v>168</v>
       </c>
       <c r="E438" t="s">
-        <v>220</v>
+        <v>168</v>
       </c>
       <c r="F438" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="439" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B439" t="s">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="C439" t="s">
-        <v>303</v>
+        <v>170</v>
       </c>
       <c r="D439" t="s">
-        <v>220</v>
+        <v>168</v>
       </c>
       <c r="E439" t="s">
-        <v>220</v>
+        <v>168</v>
       </c>
       <c r="F439" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="440" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B440" t="s">
-        <v>198</v>
+        <v>15</v>
       </c>
       <c r="C440" t="s">
-        <v>304</v>
-      </c>
-      <c r="D440" t="s">
-        <v>220</v>
-      </c>
-      <c r="E440" t="s">
-        <v>220</v>
+        <v>172</v>
       </c>
       <c r="F440" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="441" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B441" t="s">
-        <v>198</v>
+        <v>147</v>
       </c>
       <c r="C441" t="s">
-        <v>308</v>
+        <v>173</v>
       </c>
       <c r="D441" t="s">
-        <v>220</v>
+        <v>174</v>
       </c>
       <c r="E441" t="s">
-        <v>220</v>
+        <v>174</v>
       </c>
       <c r="F441" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="442" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
         <v>179</v>
       </c>
@@ -10488,19 +10407,16 @@
         <v>198</v>
       </c>
       <c r="C442" t="s">
-        <v>309</v>
+        <v>199</v>
       </c>
       <c r="D442" t="s">
-        <v>220</v>
-      </c>
-      <c r="E442" t="s">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="F442" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="443" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
         <v>179</v>
       </c>
@@ -10508,19 +10424,16 @@
         <v>198</v>
       </c>
       <c r="C443" t="s">
-        <v>311</v>
+        <v>201</v>
       </c>
       <c r="D443" t="s">
-        <v>220</v>
-      </c>
-      <c r="E443" t="s">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="F443" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="444" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
         <v>179</v>
       </c>
@@ -10528,27 +10441,24 @@
         <v>198</v>
       </c>
       <c r="C444" t="s">
-        <v>312</v>
+        <v>202</v>
       </c>
       <c r="D444" t="s">
-        <v>220</v>
-      </c>
-      <c r="E444" t="s">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="F444" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="445" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
         <v>179</v>
       </c>
       <c r="B445" t="s">
-        <v>198</v>
+        <v>218</v>
       </c>
       <c r="C445" t="s">
-        <v>313</v>
+        <v>219</v>
       </c>
       <c r="D445" t="s">
         <v>220</v>
@@ -10560,628 +10470,712 @@
         <v>12</v>
       </c>
     </row>
-    <row r="446" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
         <v>179</v>
       </c>
       <c r="B446" t="s">
+        <v>221</v>
+      </c>
+      <c r="C446" t="s">
+        <v>222</v>
+      </c>
+      <c r="D446" t="s">
+        <v>220</v>
+      </c>
+      <c r="E446" t="s">
+        <v>220</v>
+      </c>
+      <c r="F446" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="447" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A447" t="s">
+        <v>179</v>
+      </c>
+      <c r="B447" t="s">
+        <v>223</v>
+      </c>
+      <c r="C447" t="s">
+        <v>224</v>
+      </c>
+      <c r="D447" t="s">
+        <v>220</v>
+      </c>
+      <c r="E447" t="s">
+        <v>220</v>
+      </c>
+      <c r="F447" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="448" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A448" t="s">
+        <v>179</v>
+      </c>
+      <c r="B448" t="s">
+        <v>225</v>
+      </c>
+      <c r="C448" t="s">
+        <v>226</v>
+      </c>
+      <c r="D448" t="s">
+        <v>220</v>
+      </c>
+      <c r="E448" t="s">
+        <v>220</v>
+      </c>
+      <c r="F448" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="449" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A449" t="s">
+        <v>179</v>
+      </c>
+      <c r="B449" t="s">
+        <v>225</v>
+      </c>
+      <c r="C449" t="s">
+        <v>227</v>
+      </c>
+      <c r="D449" t="s">
+        <v>220</v>
+      </c>
+      <c r="E449" t="s">
+        <v>220</v>
+      </c>
+      <c r="F449" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="450" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A450" t="s">
+        <v>179</v>
+      </c>
+      <c r="B450" t="s">
+        <v>225</v>
+      </c>
+      <c r="C450" t="s">
+        <v>228</v>
+      </c>
+      <c r="D450" t="s">
+        <v>220</v>
+      </c>
+      <c r="E450" t="s">
+        <v>220</v>
+      </c>
+      <c r="F450" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="451" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A451" t="s">
+        <v>179</v>
+      </c>
+      <c r="B451" t="s">
+        <v>225</v>
+      </c>
+      <c r="C451" t="s">
+        <v>229</v>
+      </c>
+      <c r="D451" t="s">
+        <v>220</v>
+      </c>
+      <c r="E451" t="s">
+        <v>220</v>
+      </c>
+      <c r="F451" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="452" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A452" t="s">
+        <v>179</v>
+      </c>
+      <c r="B452" t="s">
+        <v>225</v>
+      </c>
+      <c r="C452" t="s">
+        <v>231</v>
+      </c>
+      <c r="D452" t="s">
+        <v>220</v>
+      </c>
+      <c r="E452" t="s">
+        <v>220</v>
+      </c>
+      <c r="F452" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="453" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A453" t="s">
+        <v>179</v>
+      </c>
+      <c r="B453" t="s">
+        <v>225</v>
+      </c>
+      <c r="C453" t="s">
+        <v>232</v>
+      </c>
+      <c r="D453" t="s">
+        <v>220</v>
+      </c>
+      <c r="E453" t="s">
+        <v>220</v>
+      </c>
+      <c r="F453" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="454" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A454" t="s">
+        <v>179</v>
+      </c>
+      <c r="B454" t="s">
+        <v>225</v>
+      </c>
+      <c r="C454" t="s">
+        <v>233</v>
+      </c>
+      <c r="D454" t="s">
+        <v>220</v>
+      </c>
+      <c r="E454" t="s">
+        <v>220</v>
+      </c>
+      <c r="F454" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="455" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A455" t="s">
+        <v>179</v>
+      </c>
+      <c r="B455" t="s">
+        <v>234</v>
+      </c>
+      <c r="C455" t="s">
+        <v>235</v>
+      </c>
+      <c r="D455" t="s">
+        <v>220</v>
+      </c>
+      <c r="E455" t="s">
+        <v>220</v>
+      </c>
+      <c r="F455" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="456" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A456" t="s">
+        <v>179</v>
+      </c>
+      <c r="B456" t="s">
+        <v>225</v>
+      </c>
+      <c r="C456" t="s">
+        <v>237</v>
+      </c>
+      <c r="D456" t="s">
+        <v>220</v>
+      </c>
+      <c r="E456" t="s">
+        <v>220</v>
+      </c>
+      <c r="F456" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="457" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A457" t="s">
+        <v>179</v>
+      </c>
+      <c r="B457" t="s">
+        <v>225</v>
+      </c>
+      <c r="C457" t="s">
+        <v>239</v>
+      </c>
+      <c r="D457" t="s">
+        <v>220</v>
+      </c>
+      <c r="E457" t="s">
+        <v>220</v>
+      </c>
+      <c r="F457" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="458" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A458" t="s">
+        <v>179</v>
+      </c>
+      <c r="B458" t="s">
+        <v>225</v>
+      </c>
+      <c r="C458" t="s">
+        <v>240</v>
+      </c>
+      <c r="D458" t="s">
+        <v>220</v>
+      </c>
+      <c r="E458" t="s">
+        <v>220</v>
+      </c>
+      <c r="F458" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="459" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A459" t="s">
+        <v>179</v>
+      </c>
+      <c r="B459" t="s">
+        <v>198</v>
+      </c>
+      <c r="C459" t="s">
+        <v>256</v>
+      </c>
+      <c r="D459" t="s">
+        <v>28</v>
+      </c>
+      <c r="F459" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="460" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A460" t="s">
+        <v>179</v>
+      </c>
+      <c r="B460" t="s">
+        <v>198</v>
+      </c>
+      <c r="C460" t="s">
+        <v>258</v>
+      </c>
+      <c r="D460" t="s">
+        <v>259</v>
+      </c>
+      <c r="E460" t="s">
+        <v>259</v>
+      </c>
+      <c r="F460" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="461" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A461" t="s">
+        <v>179</v>
+      </c>
+      <c r="B461" t="s">
+        <v>262</v>
+      </c>
+      <c r="C461" t="s">
+        <v>263</v>
+      </c>
+      <c r="D461" t="s">
+        <v>259</v>
+      </c>
+      <c r="F461" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="462" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A462" t="s">
+        <v>179</v>
+      </c>
+      <c r="B462" t="s">
+        <v>264</v>
+      </c>
+      <c r="C462" t="s">
+        <v>265</v>
+      </c>
+      <c r="D462" t="s">
+        <v>259</v>
+      </c>
+      <c r="F462" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="463" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A463" t="s">
+        <v>179</v>
+      </c>
+      <c r="B463" t="s">
         <v>205</v>
       </c>
-      <c r="C446" t="s">
-        <v>314</v>
-      </c>
-      <c r="D446" t="s">
-        <v>315</v>
-      </c>
-      <c r="F446" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="447" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A447" t="s">
-        <v>8</v>
-      </c>
-      <c r="B447" t="s">
-        <v>17</v>
-      </c>
-      <c r="C447" t="s">
-        <v>18</v>
-      </c>
-      <c r="D447" t="s">
-        <v>11</v>
-      </c>
-      <c r="G447" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="448" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A448" t="s">
-        <v>8</v>
-      </c>
-      <c r="B448" t="s">
-        <v>38</v>
-      </c>
-      <c r="C448" t="s">
-        <v>40</v>
-      </c>
-      <c r="D448" t="s">
-        <v>41</v>
-      </c>
-      <c r="E448" t="s">
-        <v>37</v>
-      </c>
-      <c r="F448" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="449" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A449" t="s">
-        <v>8</v>
-      </c>
-      <c r="B449" t="s">
-        <v>26</v>
-      </c>
-      <c r="C449" t="s">
-        <v>42</v>
-      </c>
-      <c r="D449" t="s">
-        <v>37</v>
-      </c>
-      <c r="E449" t="s">
-        <v>37</v>
-      </c>
-      <c r="F449" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="450" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A450" t="s">
-        <v>8</v>
-      </c>
-      <c r="B450" t="s">
-        <v>26</v>
-      </c>
-      <c r="C450" t="s">
-        <v>43</v>
-      </c>
-      <c r="D450" t="s">
-        <v>41</v>
-      </c>
-      <c r="E450" t="s">
-        <v>37</v>
-      </c>
-      <c r="F450" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="451" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A451" t="s">
-        <v>8</v>
-      </c>
-      <c r="B451" t="s">
-        <v>9</v>
-      </c>
-      <c r="C451" t="s">
-        <v>53</v>
-      </c>
-      <c r="D451" t="s">
-        <v>11</v>
-      </c>
-      <c r="G451" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="452" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A452" t="s">
-        <v>8</v>
-      </c>
-      <c r="B452" t="s">
-        <v>26</v>
-      </c>
-      <c r="C452" t="s">
-        <v>57</v>
-      </c>
-      <c r="D452" t="s">
-        <v>56</v>
-      </c>
-      <c r="F452" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="453" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A453" t="s">
-        <v>8</v>
-      </c>
-      <c r="B453" t="s">
-        <v>35</v>
-      </c>
-      <c r="C453" t="s">
-        <v>58</v>
-      </c>
-      <c r="D453" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="454" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A454" t="s">
-        <v>8</v>
-      </c>
-      <c r="B454" t="s">
-        <v>38</v>
-      </c>
-      <c r="C454" t="s">
-        <v>60</v>
-      </c>
-      <c r="D454" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="455" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A455" t="s">
-        <v>8</v>
-      </c>
-      <c r="B455" t="s">
-        <v>26</v>
-      </c>
-      <c r="C455" t="s">
-        <v>61</v>
-      </c>
-      <c r="D455" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="456" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A456" t="s">
-        <v>8</v>
-      </c>
-      <c r="B456" t="s">
-        <v>66</v>
-      </c>
-      <c r="C456" t="s">
-        <v>67</v>
-      </c>
-      <c r="D456" t="s">
-        <v>28</v>
-      </c>
-      <c r="F456" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="457" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A457" t="s">
-        <v>8</v>
-      </c>
-      <c r="B457" t="s">
-        <v>17</v>
-      </c>
-      <c r="C457" t="s">
-        <v>75</v>
-      </c>
-      <c r="D457" t="s">
-        <v>11</v>
-      </c>
-      <c r="G457" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="458" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A458" t="s">
-        <v>8</v>
-      </c>
-      <c r="B458" t="s">
-        <v>17</v>
-      </c>
-      <c r="C458" t="s">
-        <v>77</v>
-      </c>
-      <c r="D458" t="s">
-        <v>11</v>
-      </c>
-      <c r="G458" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="459" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A459" t="s">
-        <v>8</v>
-      </c>
-      <c r="B459" t="s">
-        <v>17</v>
-      </c>
-      <c r="C459" t="s">
-        <v>82</v>
-      </c>
-      <c r="D459" t="s">
-        <v>11</v>
-      </c>
-      <c r="G459" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="460" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A460" t="s">
-        <v>8</v>
-      </c>
-      <c r="B460" t="s">
-        <v>88</v>
-      </c>
-      <c r="C460" t="s">
-        <v>89</v>
-      </c>
-      <c r="D460" t="s">
-        <v>11</v>
-      </c>
-      <c r="G460" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="461" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A461" t="s">
-        <v>8</v>
-      </c>
-      <c r="B461" t="s">
-        <v>88</v>
-      </c>
-      <c r="C461" t="s">
-        <v>97</v>
-      </c>
-      <c r="D461" t="s">
-        <v>11</v>
-      </c>
-      <c r="G461" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="462" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A462" t="s">
-        <v>8</v>
-      </c>
-      <c r="B462" t="s">
-        <v>17</v>
-      </c>
-      <c r="C462" t="s">
-        <v>101</v>
-      </c>
-      <c r="D462" t="s">
-        <v>11</v>
-      </c>
-      <c r="G462" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="463" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A463" t="s">
-        <v>8</v>
-      </c>
-      <c r="B463" t="s">
-        <v>17</v>
-      </c>
       <c r="C463" t="s">
-        <v>106</v>
+        <v>266</v>
       </c>
       <c r="D463" t="s">
-        <v>11</v>
-      </c>
-      <c r="G463" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="464" spans="1:7" x14ac:dyDescent="0.25">
+        <v>259</v>
+      </c>
+      <c r="F463" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="464" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="B464" t="s">
-        <v>17</v>
+        <v>264</v>
       </c>
       <c r="C464" t="s">
-        <v>114</v>
+        <v>267</v>
       </c>
       <c r="D464" t="s">
-        <v>11</v>
-      </c>
-      <c r="G464" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="465" spans="1:7" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+      <c r="E464" t="s">
+        <v>268</v>
+      </c>
+      <c r="F464" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="465" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="B465" t="s">
-        <v>88</v>
+        <v>205</v>
       </c>
       <c r="C465" t="s">
-        <v>126</v>
+        <v>269</v>
       </c>
       <c r="D465" t="s">
-        <v>11</v>
-      </c>
-      <c r="G465" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="466" spans="1:7" x14ac:dyDescent="0.25">
+        <v>259</v>
+      </c>
+      <c r="F465" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="466" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="B466" t="s">
-        <v>17</v>
+        <v>205</v>
       </c>
       <c r="C466" t="s">
-        <v>130</v>
+        <v>270</v>
       </c>
       <c r="D466" t="s">
-        <v>11</v>
-      </c>
-      <c r="G466" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="467" spans="1:7" x14ac:dyDescent="0.25">
+        <v>271</v>
+      </c>
+      <c r="E466" t="s">
+        <v>271</v>
+      </c>
+      <c r="F466" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="467" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="B467" t="s">
-        <v>88</v>
+        <v>262</v>
       </c>
       <c r="C467" t="s">
-        <v>133</v>
+        <v>285</v>
       </c>
       <c r="D467" t="s">
-        <v>11</v>
-      </c>
-      <c r="G467" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="468" spans="1:7" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+      <c r="E467" t="s">
+        <v>268</v>
+      </c>
+      <c r="F467" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="468" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="B468" t="s">
-        <v>17</v>
+        <v>264</v>
       </c>
       <c r="C468" t="s">
-        <v>141</v>
+        <v>287</v>
       </c>
       <c r="D468" t="s">
-        <v>11</v>
-      </c>
-      <c r="G468" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="469" spans="1:7" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+      <c r="E468" t="s">
+        <v>288</v>
+      </c>
+      <c r="F468" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="469" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="B469" t="s">
-        <v>88</v>
+        <v>262</v>
       </c>
       <c r="C469" t="s">
-        <v>146</v>
+        <v>289</v>
       </c>
       <c r="D469" t="s">
-        <v>11</v>
-      </c>
-      <c r="G469" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="470" spans="1:7" x14ac:dyDescent="0.25">
+        <v>268</v>
+      </c>
+      <c r="E469" t="s">
+        <v>268</v>
+      </c>
+      <c r="F469" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="470" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="B470" t="s">
-        <v>88</v>
+        <v>264</v>
       </c>
       <c r="C470" t="s">
-        <v>158</v>
+        <v>291</v>
       </c>
       <c r="D470" t="s">
-        <v>11</v>
-      </c>
-      <c r="G470" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="471" spans="1:7" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+      <c r="E470" t="s">
+        <v>288</v>
+      </c>
+      <c r="F470" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="471" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="B471" t="s">
-        <v>26</v>
+        <v>262</v>
       </c>
       <c r="C471" t="s">
-        <v>161</v>
+        <v>292</v>
       </c>
       <c r="D471" t="s">
-        <v>162</v>
+        <v>293</v>
+      </c>
+      <c r="E471" t="s">
+        <v>293</v>
       </c>
       <c r="F471" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="472" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="B472" t="s">
-        <v>26</v>
+        <v>264</v>
       </c>
       <c r="C472" t="s">
-        <v>171</v>
+        <v>294</v>
       </c>
       <c r="D472" t="s">
-        <v>168</v>
+        <v>293</v>
+      </c>
+      <c r="E472" t="s">
+        <v>293</v>
       </c>
       <c r="F472" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="473" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="B473" t="s">
-        <v>17</v>
+        <v>198</v>
       </c>
       <c r="C473" t="s">
-        <v>177</v>
+        <v>296</v>
       </c>
       <c r="D473" t="s">
-        <v>11</v>
-      </c>
-      <c r="G473" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="474" spans="1:7" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="E473" t="s">
+        <v>220</v>
+      </c>
+      <c r="F473" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="474" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
         <v>179</v>
       </c>
       <c r="B474" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="C474" t="s">
-        <v>186</v>
+        <v>302</v>
       </c>
       <c r="D474" t="s">
-        <v>11</v>
-      </c>
-      <c r="G474" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="475" spans="1:7" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="E474" t="s">
+        <v>220</v>
+      </c>
+      <c r="F474" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="475" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
         <v>179</v>
       </c>
       <c r="B475" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="C475" t="s">
-        <v>189</v>
+        <v>303</v>
       </c>
       <c r="D475" t="s">
-        <v>11</v>
-      </c>
-      <c r="G475" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="476" spans="1:7" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="E475" t="s">
+        <v>220</v>
+      </c>
+      <c r="F475" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="476" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
         <v>179</v>
       </c>
       <c r="B476" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="C476" t="s">
-        <v>192</v>
+        <v>304</v>
       </c>
       <c r="D476" t="s">
-        <v>11</v>
-      </c>
-      <c r="G476" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="477" spans="1:7" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="E476" t="s">
+        <v>220</v>
+      </c>
+      <c r="F476" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="477" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
         <v>179</v>
       </c>
       <c r="B477" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="C477" t="s">
-        <v>196</v>
+        <v>308</v>
       </c>
       <c r="D477" t="s">
-        <v>11</v>
-      </c>
-      <c r="G477" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="478" spans="1:7" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="E477" t="s">
+        <v>220</v>
+      </c>
+      <c r="F477" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="478" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
         <v>179</v>
       </c>
       <c r="B478" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="C478" t="s">
-        <v>197</v>
+        <v>309</v>
       </c>
       <c r="D478" t="s">
-        <v>11</v>
-      </c>
-      <c r="G478" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="479" spans="1:7" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="E478" t="s">
+        <v>220</v>
+      </c>
+      <c r="F478" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="479" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
         <v>179</v>
       </c>
       <c r="B479" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="C479" t="s">
-        <v>206</v>
+        <v>311</v>
       </c>
       <c r="D479" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="E479" t="s">
-        <v>288</v>
+        <v>220</v>
       </c>
       <c r="F479" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="480" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
         <v>179</v>
       </c>
       <c r="B480" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="C480" t="s">
-        <v>208</v>
+        <v>312</v>
       </c>
       <c r="D480" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="E480" t="s">
-        <v>288</v>
+        <v>220</v>
       </c>
       <c r="F480" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="481" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
         <v>179</v>
       </c>
       <c r="B481" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="C481" t="s">
-        <v>209</v>
+        <v>313</v>
       </c>
       <c r="D481" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="E481" t="s">
-        <v>288</v>
+        <v>220</v>
       </c>
       <c r="F481" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="482" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A482" t="s">
         <v>179</v>
       </c>
@@ -11189,357 +11183,384 @@
         <v>205</v>
       </c>
       <c r="C482" t="s">
+        <v>314</v>
+      </c>
+      <c r="D482" t="s">
+        <v>315</v>
+      </c>
+      <c r="F482" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="483" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A483" t="s">
+        <v>8</v>
+      </c>
+      <c r="B483" t="s">
+        <v>38</v>
+      </c>
+      <c r="C483" t="s">
+        <v>40</v>
+      </c>
+      <c r="D483" t="s">
+        <v>41</v>
+      </c>
+      <c r="E483" t="s">
+        <v>37</v>
+      </c>
+      <c r="F483" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="484" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A484" t="s">
+        <v>8</v>
+      </c>
+      <c r="B484" t="s">
+        <v>26</v>
+      </c>
+      <c r="C484" t="s">
+        <v>42</v>
+      </c>
+      <c r="D484" t="s">
+        <v>37</v>
+      </c>
+      <c r="E484" t="s">
+        <v>37</v>
+      </c>
+      <c r="F484" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="485" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A485" t="s">
+        <v>8</v>
+      </c>
+      <c r="B485" t="s">
+        <v>26</v>
+      </c>
+      <c r="C485" t="s">
+        <v>43</v>
+      </c>
+      <c r="D485" t="s">
+        <v>41</v>
+      </c>
+      <c r="E485" t="s">
+        <v>37</v>
+      </c>
+      <c r="F485" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="486" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A486" t="s">
+        <v>8</v>
+      </c>
+      <c r="B486" t="s">
+        <v>26</v>
+      </c>
+      <c r="C486" t="s">
+        <v>57</v>
+      </c>
+      <c r="D486" t="s">
+        <v>56</v>
+      </c>
+      <c r="F486" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="487" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A487" t="s">
+        <v>8</v>
+      </c>
+      <c r="B487" t="s">
+        <v>66</v>
+      </c>
+      <c r="C487" t="s">
+        <v>67</v>
+      </c>
+      <c r="D487" t="s">
+        <v>28</v>
+      </c>
+      <c r="F487" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="488" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A488" t="s">
+        <v>8</v>
+      </c>
+      <c r="B488" t="s">
+        <v>26</v>
+      </c>
+      <c r="C488" t="s">
+        <v>161</v>
+      </c>
+      <c r="D488" t="s">
+        <v>162</v>
+      </c>
+      <c r="F488" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="489" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A489" t="s">
+        <v>8</v>
+      </c>
+      <c r="B489" t="s">
+        <v>26</v>
+      </c>
+      <c r="C489" t="s">
+        <v>171</v>
+      </c>
+      <c r="D489" t="s">
+        <v>168</v>
+      </c>
+      <c r="F489" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="490" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A490" t="s">
+        <v>179</v>
+      </c>
+      <c r="B490" t="s">
+        <v>205</v>
+      </c>
+      <c r="C490" t="s">
+        <v>206</v>
+      </c>
+      <c r="D490" t="s">
+        <v>207</v>
+      </c>
+      <c r="E490" t="s">
+        <v>288</v>
+      </c>
+      <c r="F490" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="491" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A491" t="s">
+        <v>179</v>
+      </c>
+      <c r="B491" t="s">
+        <v>205</v>
+      </c>
+      <c r="C491" t="s">
+        <v>208</v>
+      </c>
+      <c r="D491" t="s">
+        <v>207</v>
+      </c>
+      <c r="E491" t="s">
+        <v>288</v>
+      </c>
+      <c r="F491" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="492" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A492" t="s">
+        <v>179</v>
+      </c>
+      <c r="B492" t="s">
+        <v>205</v>
+      </c>
+      <c r="C492" t="s">
+        <v>209</v>
+      </c>
+      <c r="D492" t="s">
+        <v>207</v>
+      </c>
+      <c r="E492" t="s">
+        <v>288</v>
+      </c>
+      <c r="F492" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="493" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A493" t="s">
+        <v>179</v>
+      </c>
+      <c r="B493" t="s">
+        <v>205</v>
+      </c>
+      <c r="C493" t="s">
         <v>210</v>
       </c>
-      <c r="D482" t="s">
+      <c r="D493" t="s">
         <v>207</v>
       </c>
-      <c r="E482" t="s">
+      <c r="E493" t="s">
         <v>288</v>
       </c>
-      <c r="F482" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="483" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A483" t="s">
-        <v>179</v>
-      </c>
-      <c r="B483" t="s">
+      <c r="F493" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="494" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A494" t="s">
+        <v>179</v>
+      </c>
+      <c r="B494" t="s">
         <v>205</v>
       </c>
-      <c r="C483" t="s">
+      <c r="C494" t="s">
         <v>211</v>
       </c>
-      <c r="D483" t="s">
+      <c r="D494" t="s">
         <v>207</v>
       </c>
-      <c r="E483" t="s">
+      <c r="E494" t="s">
         <v>288</v>
       </c>
-      <c r="F483" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="484" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A484" t="s">
-        <v>179</v>
-      </c>
-      <c r="B484" t="s">
+      <c r="F494" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="495" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A495" t="s">
+        <v>179</v>
+      </c>
+      <c r="B495" t="s">
         <v>205</v>
       </c>
-      <c r="C484" t="s">
+      <c r="C495" t="s">
         <v>212</v>
       </c>
-      <c r="D484" t="s">
+      <c r="D495" t="s">
         <v>207</v>
       </c>
-      <c r="E484" t="s">
+      <c r="E495" t="s">
         <v>288</v>
       </c>
-      <c r="F484" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="485" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A485" t="s">
-        <v>179</v>
-      </c>
-      <c r="B485" t="s">
-        <v>203</v>
-      </c>
-      <c r="C485" t="s">
-        <v>215</v>
-      </c>
-      <c r="D485" t="s">
-        <v>11</v>
-      </c>
-      <c r="G485" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="486" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A486" t="s">
-        <v>179</v>
-      </c>
-      <c r="B486" t="s">
+      <c r="F495" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="496" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A496" t="s">
+        <v>179</v>
+      </c>
+      <c r="B496" t="s">
         <v>225</v>
       </c>
-      <c r="C486" t="s">
+      <c r="C496" t="s">
         <v>230</v>
       </c>
-      <c r="D486" t="s">
+      <c r="D496" t="s">
         <v>59</v>
       </c>
-      <c r="E486" t="s">
+      <c r="E496" t="s">
         <v>220</v>
       </c>
-      <c r="F486" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="487" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A487" t="s">
-        <v>179</v>
-      </c>
-      <c r="B487" t="s">
+      <c r="F496" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="497" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A497" t="s">
+        <v>179</v>
+      </c>
+      <c r="B497" t="s">
         <v>225</v>
       </c>
-      <c r="C487" t="s">
+      <c r="C497" t="s">
         <v>236</v>
       </c>
-      <c r="D487" t="s">
+      <c r="D497" t="s">
         <v>59</v>
       </c>
-      <c r="E487" t="s">
+      <c r="E497" t="s">
         <v>220</v>
       </c>
-      <c r="F487" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="488" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A488" t="s">
-        <v>179</v>
-      </c>
-      <c r="B488" t="s">
+      <c r="F497" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="498" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A498" t="s">
+        <v>179</v>
+      </c>
+      <c r="B498" t="s">
         <v>234</v>
       </c>
-      <c r="C488" t="s">
+      <c r="C498" t="s">
         <v>238</v>
       </c>
-      <c r="D488" t="s">
+      <c r="D498" t="s">
         <v>59</v>
       </c>
-      <c r="E488" t="s">
+      <c r="E498" t="s">
         <v>220</v>
       </c>
-      <c r="F488" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="489" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A489" t="s">
-        <v>179</v>
-      </c>
-      <c r="B489" t="s">
-        <v>203</v>
-      </c>
-      <c r="C489" t="s">
-        <v>242</v>
-      </c>
-      <c r="D489" t="s">
-        <v>11</v>
-      </c>
-      <c r="G489" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="490" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A490" t="s">
-        <v>179</v>
-      </c>
-      <c r="B490" t="s">
-        <v>182</v>
-      </c>
-      <c r="C490" t="s">
-        <v>246</v>
-      </c>
-      <c r="D490" t="s">
-        <v>11</v>
-      </c>
-      <c r="G490" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="491" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A491" t="s">
-        <v>179</v>
-      </c>
-      <c r="B491" t="s">
-        <v>182</v>
-      </c>
-      <c r="C491" t="s">
-        <v>247</v>
-      </c>
-      <c r="D491" t="s">
-        <v>11</v>
-      </c>
-      <c r="G491" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="492" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A492" t="s">
-        <v>179</v>
-      </c>
-      <c r="B492" t="s">
-        <v>182</v>
-      </c>
-      <c r="C492" t="s">
-        <v>250</v>
-      </c>
-      <c r="D492" t="s">
-        <v>11</v>
-      </c>
-      <c r="G492" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="493" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A493" t="s">
-        <v>179</v>
-      </c>
-      <c r="B493" t="s">
-        <v>180</v>
-      </c>
-      <c r="C493" t="s">
-        <v>252</v>
-      </c>
-      <c r="D493" t="s">
-        <v>11</v>
-      </c>
-      <c r="G493" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="494" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A494" t="s">
-        <v>179</v>
-      </c>
-      <c r="B494" t="s">
-        <v>182</v>
-      </c>
-      <c r="C494" t="s">
-        <v>253</v>
-      </c>
-      <c r="D494" t="s">
-        <v>11</v>
-      </c>
-      <c r="G494" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="495" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A495" t="s">
-        <v>179</v>
-      </c>
-      <c r="B495" t="s">
-        <v>182</v>
-      </c>
-      <c r="C495" t="s">
-        <v>255</v>
-      </c>
-      <c r="D495" t="s">
-        <v>11</v>
-      </c>
-      <c r="G495" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="496" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A496" t="s">
-        <v>179</v>
-      </c>
-      <c r="B496" t="s">
-        <v>182</v>
-      </c>
-      <c r="C496" t="s">
-        <v>276</v>
-      </c>
-      <c r="D496" t="s">
-        <v>11</v>
-      </c>
-      <c r="G496" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="497" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A497" t="s">
-        <v>179</v>
-      </c>
-      <c r="B497" t="s">
-        <v>182</v>
-      </c>
-      <c r="C497" t="s">
-        <v>279</v>
-      </c>
-      <c r="D497" t="s">
-        <v>11</v>
-      </c>
-      <c r="G497" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="498" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A498" t="s">
-        <v>179</v>
-      </c>
-      <c r="B498" t="s">
-        <v>203</v>
-      </c>
-      <c r="C498" t="s">
-        <v>280</v>
-      </c>
-      <c r="D498" t="s">
-        <v>11</v>
-      </c>
-      <c r="G498" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="499" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F498" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="499" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A499" t="s">
         <v>179</v>
       </c>
       <c r="B499" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C499" t="s">
-        <v>282</v>
+        <v>297</v>
       </c>
       <c r="D499" t="s">
-        <v>11</v>
-      </c>
-      <c r="G499" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="500" spans="1:7" x14ac:dyDescent="0.25">
+        <v>298</v>
+      </c>
+      <c r="E499" t="s">
+        <v>220</v>
+      </c>
+      <c r="F499" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="500" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A500" t="s">
         <v>179</v>
       </c>
       <c r="B500" t="s">
-        <v>264</v>
+        <v>198</v>
       </c>
       <c r="C500" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="D500" t="s">
-        <v>207</v>
-      </c>
-      <c r="G500" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="501" spans="1:7" x14ac:dyDescent="0.25">
+        <v>298</v>
+      </c>
+      <c r="E500" t="s">
+        <v>220</v>
+      </c>
+      <c r="F500" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="501" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A501" t="s">
         <v>179</v>
       </c>
       <c r="B501" t="s">
-        <v>264</v>
+        <v>198</v>
       </c>
       <c r="C501" t="s">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="D501" t="s">
-        <v>268</v>
-      </c>
-      <c r="G501" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="502" spans="1:7" x14ac:dyDescent="0.25">
+        <v>298</v>
+      </c>
+      <c r="E501" t="s">
+        <v>220</v>
+      </c>
+      <c r="F501" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="502" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A502" t="s">
         <v>179</v>
       </c>
@@ -11547,7 +11568,7 @@
         <v>198</v>
       </c>
       <c r="C502" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="D502" t="s">
         <v>298</v>
@@ -11559,15 +11580,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="503" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="503" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A503" t="s">
         <v>179</v>
       </c>
       <c r="B503" t="s">
-        <v>198</v>
+        <v>305</v>
       </c>
       <c r="C503" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="D503" t="s">
         <v>298</v>
@@ -11579,7 +11600,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="504" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="504" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A504" t="s">
         <v>179</v>
       </c>
@@ -11587,7 +11608,7 @@
         <v>198</v>
       </c>
       <c r="C504" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="D504" t="s">
         <v>298</v>
@@ -11599,7 +11620,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="505" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="505" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A505" t="s">
         <v>179</v>
       </c>
@@ -11607,7 +11628,7 @@
         <v>198</v>
       </c>
       <c r="C505" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="D505" t="s">
         <v>298</v>
@@ -11619,18 +11640,18 @@
         <v>12</v>
       </c>
     </row>
-    <row r="506" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="506" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A506" t="s">
         <v>179</v>
       </c>
       <c r="B506" t="s">
-        <v>305</v>
+        <v>205</v>
       </c>
       <c r="C506" t="s">
-        <v>306</v>
+        <v>316</v>
       </c>
       <c r="D506" t="s">
-        <v>298</v>
+        <v>315</v>
       </c>
       <c r="E506" t="s">
         <v>220</v>
@@ -11639,64 +11660,46 @@
         <v>12</v>
       </c>
     </row>
-    <row r="507" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="507" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A507" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B507" t="s">
-        <v>198</v>
+        <v>35</v>
       </c>
       <c r="C507" t="s">
-        <v>307</v>
+        <v>58</v>
       </c>
       <c r="D507" t="s">
-        <v>298</v>
-      </c>
-      <c r="E507" t="s">
-        <v>220</v>
-      </c>
-      <c r="F507" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="508" spans="1:7" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="508" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A508" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B508" t="s">
-        <v>198</v>
+        <v>38</v>
       </c>
       <c r="C508" t="s">
-        <v>310</v>
+        <v>60</v>
       </c>
       <c r="D508" t="s">
-        <v>298</v>
-      </c>
-      <c r="E508" t="s">
-        <v>220</v>
-      </c>
-      <c r="F508" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="509" spans="1:7" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="509" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A509" t="s">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="B509" t="s">
-        <v>205</v>
+        <v>26</v>
       </c>
       <c r="C509" t="s">
-        <v>316</v>
+        <v>61</v>
       </c>
       <c r="D509" t="s">
-        <v>315</v>
-      </c>
-      <c r="E509" t="s">
-        <v>220</v>
-      </c>
-      <c r="F509" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gem mine valg (sport + danske backdrops) 2026-10-05 21:38:16
</commit_message>
<xml_diff>
--- a/data/sport_artwork_review.xlsx
+++ b/data/sport_artwork_review.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EPGoal\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9930A843-9C8A-4B2A-9BE1-EC59E1969962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3EF558C-5572-47A6-8C94-9EC5B90C83EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sport-artwork review" sheetId="1" r:id="rId1"/>
     <sheet name="BilledeListe" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet name="Forsvundne (havde valg)" sheetId="3" r:id="rId3"/>
-    <sheet name="Vejledning" sheetId="4" r:id="rId4"/>
+    <sheet name="Vejledning" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sport-artwork review'!$A$1:$H$1</definedName>
@@ -27,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1109" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="894" uniqueCount="334">
   <si>
     <t>Kanalgruppe</t>
   </si>
@@ -65,66 +64,63 @@
     <t>(intet billede)</t>
   </si>
   <si>
+    <t>Faster</t>
+  </si>
+  <si>
+    <t>Forsvundet sporløst</t>
+  </si>
+  <si>
+    <t>Gridiron Gang</t>
+  </si>
+  <si>
+    <t>Hawaii Five-0</t>
+  </si>
+  <si>
+    <t>Jane Got a Gun</t>
+  </si>
+  <si>
+    <t>Last Light</t>
+  </si>
+  <si>
+    <t>NCIS</t>
+  </si>
+  <si>
+    <t>NCIS: Los Angeles</t>
+  </si>
+  <si>
+    <t>Pacific Blue</t>
+  </si>
+  <si>
+    <t>S.W.A.T.</t>
+  </si>
+  <si>
+    <t>Shipping Wars</t>
+  </si>
+  <si>
+    <t>Snitch</t>
+  </si>
+  <si>
+    <t>The Man Who Stole The Scream</t>
+  </si>
+  <si>
+    <t>Walking Tall</t>
+  </si>
+  <si>
+    <t>We Got This</t>
+  </si>
+  <si>
+    <t>C - DR1/DR2</t>
+  </si>
+  <si>
+    <t>DR1.dk</t>
+  </si>
+  <si>
+    <t>Aftenshowet</t>
+  </si>
+  <si>
     <t>X</t>
   </si>
   <si>
-    <t>Faster</t>
-  </si>
-  <si>
-    <t>Forsvundet sporløst</t>
-  </si>
-  <si>
-    <t>Gridiron Gang</t>
-  </si>
-  <si>
-    <t>Hawaii Five-0</t>
-  </si>
-  <si>
-    <t>Jane Got a Gun</t>
-  </si>
-  <si>
-    <t>Last Light</t>
-  </si>
-  <si>
-    <t>NCIS</t>
-  </si>
-  <si>
-    <t>NCIS: Los Angeles</t>
-  </si>
-  <si>
-    <t>Pacific Blue</t>
-  </si>
-  <si>
-    <t>S.W.A.T.</t>
-  </si>
-  <si>
-    <t>Shipping Wars</t>
-  </si>
-  <si>
-    <t>Snitch</t>
-  </si>
-  <si>
-    <t>The Man Who Stole The Scream</t>
-  </si>
-  <si>
-    <t>Walking Tall</t>
-  </si>
-  <si>
-    <t>We Got This</t>
-  </si>
-  <si>
-    <t>C - DR1/DR2</t>
-  </si>
-  <si>
-    <t>DR1.dk</t>
-  </si>
-  <si>
-    <t>Aftenshowet</t>
-  </si>
-  <si>
-    <t>TMDb</t>
-  </si>
-  <si>
     <t>Alene i vildmarken Australien</t>
   </si>
   <si>
@@ -194,6 +190,9 @@
     <t>Deadline: Kampen om elbilerne</t>
   </si>
   <si>
+    <t>Deadline: Må en anklager bære tørklæde?</t>
+  </si>
+  <si>
     <t>Debatten</t>
   </si>
   <si>
@@ -972,231 +971,6 @@
   </si>
   <si>
     <t>tv3sport-generic.jpg</t>
-  </si>
-  <si>
-    <t>Tidligere valgt billede</t>
-  </si>
-  <si>
-    <t>Danskerklubben</t>
-  </si>
-  <si>
-    <t>Darts: World Grand Prix</t>
-  </si>
-  <si>
-    <t>EHF European League</t>
-  </si>
-  <si>
-    <t>EHF European League: Karvina-TTH Holstebro (m)</t>
-  </si>
-  <si>
-    <t>EHF European League: Mors - Thy - MOL Tatabanya</t>
-  </si>
-  <si>
-    <t>EHF Men's European League: HCB Karvina - TTH Holstebro</t>
-  </si>
-  <si>
-    <t>EHF Men's European League: Mors-Thy - MOL Tatabanya</t>
-  </si>
-  <si>
-    <t>EHF Women's Champions League</t>
-  </si>
-  <si>
-    <t>EHF Women's Champions League: Odense Håndbold - Storhamar</t>
-  </si>
-  <si>
-    <t>EHF Women's Champions League: Odense-Storhamar (k)</t>
-  </si>
-  <si>
-    <t>EHF Women's Champions League: Team Esbjerg - Buducnost</t>
-  </si>
-  <si>
-    <t>EHF Women's Champions League: Team Esbjerg-Buducnost (k)</t>
-  </si>
-  <si>
-    <t>F1: Bahrains Grand Prix - Løbet</t>
-  </si>
-  <si>
-    <t>Formel 1: Bahrains Grand Prix</t>
-  </si>
-  <si>
-    <t>Formel 1: Studiet</t>
-  </si>
-  <si>
-    <t>NHL</t>
-  </si>
-  <si>
-    <t>NHL: New York Rangers - Utah Mammoth</t>
-  </si>
-  <si>
-    <t>NHL: Tampa Bay Lightning - Philadelphia Flyers</t>
-  </si>
-  <si>
-    <t>NHL: Tampa Bay-Philadelphia</t>
-  </si>
-  <si>
-    <t>Sportstalk: Sportstalk: Ronaldos uværdige exit</t>
-  </si>
-  <si>
-    <t>TV-Udbruddet</t>
-  </si>
-  <si>
-    <t>TV-Udbruddet: TV - udbruddet</t>
-  </si>
-  <si>
-    <t>Watt the F1!?</t>
-  </si>
-  <si>
-    <t>B - TV2 Sport/TV2 Sport X/TV2</t>
-  </si>
-  <si>
-    <t>ATP: Alcaraz-Shapovalov, kvartfinale, Tokyo</t>
-  </si>
-  <si>
-    <t>ATP: Kvartfinaler, Beijing</t>
-  </si>
-  <si>
-    <t>ATP: Semifinale, Beijing</t>
-  </si>
-  <si>
-    <t>ATP: Semifinale, Tokyo</t>
-  </si>
-  <si>
-    <t>ATP: Vacherot-Fils, kvartfinale, Tokyo</t>
-  </si>
-  <si>
-    <t>ATP: Zverev-Djokovic, kvartfinale, Beijing</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League - Det bedste fra dagen</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League - Studie</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League - Studie: UEFA Nations League: Studiet</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: Rumænien-Sverige</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: Bosnien-Hercegovina - Polen</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: Cypern-Letland</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: England-Tjekkiet</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: Frankrig-Belgien</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: Grækenland-Tyskland</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: Holland-Serbien</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: Italien-Tyrkiet</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: Kasakhstan-Færøerne</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: Kosovo-Østrig</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: Kroatien-Spanien</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: Portugal-Norge</t>
-  </si>
-  <si>
-    <t>Fodbold: Nations League: UEFA Nations League: Wales-Danmark</t>
-  </si>
-  <si>
-    <t>Mads Pedersens grønne Tour-triumf</t>
-  </si>
-  <si>
-    <t>NFL: NFL: Washington Commanders-Indianapolis Colts</t>
-  </si>
-  <si>
-    <t>Tennis ATP 500.jpg</t>
-  </si>
-  <si>
-    <t>NFL: Washington Commanders-Indianapolis Colts</t>
-  </si>
-  <si>
-    <t>Tennis: ATP - Tokyo</t>
-  </si>
-  <si>
-    <t>Tennis: ATP - Tokyo: ATP: Semifinale, Tokyo</t>
-  </si>
-  <si>
-    <t>Tennis: ATP 500 - Beijing - Kampe</t>
-  </si>
-  <si>
-    <t>Tennis: ATP 500 - Beijing - Kampe: ATP: Semifinale, Beijing</t>
-  </si>
-  <si>
-    <t>Tennis: WTA 1000 - Beijng - Kampe</t>
-  </si>
-  <si>
-    <t>Tennis: WTA 1000 - Beijng - Kampe: WTA: Beijing</t>
-  </si>
-  <si>
-    <t>UEFA Nations League - Det bedste fra dagen</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Aserbajdsjan-Litauen</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Bosnien-Hercegovina - Polen</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Cypern-Letland</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Frankrig-Belgien</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Før Wales-Danmark</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Grækenland-Tyskland</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Holland-Serbien</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Italien-Tyrkiet</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Kosovo-Østrig</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Kroatien-England</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Portugal-Norge</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Rumænien-Sverige</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Spanien-Tjekkiet</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Studiet</t>
-  </si>
-  <si>
-    <t>UEFA Nations League: Wales-Danmark</t>
-  </si>
-  <si>
-    <t>WTA: Muchova-Samsonova, Beijing</t>
   </si>
   <si>
     <t>Sådan bruger du denne fil</t>
@@ -1618,7 +1392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H141"/>
+  <dimension ref="A1:H142"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1658,2391 +1432,2412 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>
       </c>
       <c r="G3" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="G4" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
       </c>
       <c r="G5" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="G6" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="G7" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
       </c>
       <c r="G8" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
       </c>
       <c r="G9" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="G10" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="G11" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
       </c>
       <c r="G12" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
       </c>
       <c r="G13" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B14" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
       </c>
       <c r="G14" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C15" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
       </c>
       <c r="G15" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B16" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
       <c r="G16" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="C17" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
       </c>
       <c r="G17" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G18" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C19" t="s">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="D19" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G19" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G20" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C21" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="D21" t="s">
         <v>11</v>
       </c>
       <c r="G21" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C22" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
       </c>
       <c r="G22" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C23" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="D23" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G23" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="C24" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="G24" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C25" t="s">
-        <v>39</v>
+        <v>55</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G25" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C26" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="G26" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="G27" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="G28" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C29" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="D29" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G29" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B30" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C30" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
       </c>
       <c r="G30" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B31" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
       </c>
       <c r="G31" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B32" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C32" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="D32" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G32" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C33" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="D33" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G33" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B34" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C34" t="s">
-        <v>48</v>
+        <v>64</v>
       </c>
       <c r="D34" t="s">
         <v>11</v>
       </c>
       <c r="G34" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C35" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="D35" t="s">
         <v>11</v>
       </c>
       <c r="G35" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B36" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="C36" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="D36" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G36" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B37" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C37" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
       <c r="G37" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B38" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C38" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="G38" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B39" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C39" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="G39" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C40" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="D40" t="s">
         <v>11</v>
       </c>
       <c r="G40" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B41" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C41" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="D41" t="s">
         <v>11</v>
       </c>
       <c r="G41" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B42" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C42" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="D42" t="s">
         <v>11</v>
       </c>
       <c r="G42" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B43" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C43" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="D43" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G43" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B44" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C44" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="D44" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G44" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B45" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C45" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="D45" t="s">
         <v>11</v>
       </c>
       <c r="G45" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B46" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C46" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="D46" t="s">
         <v>11</v>
       </c>
       <c r="G46" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B47" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C47" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="D47" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G47" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B48" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C48" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="D48" t="s">
         <v>11</v>
       </c>
       <c r="G48" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B49" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C49" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D49" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G49" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B50" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C50" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="D50" t="s">
         <v>11</v>
       </c>
       <c r="G50" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B51" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C51" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="D51" t="s">
         <v>11</v>
       </c>
       <c r="G51" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B52" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C52" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="D52" t="s">
         <v>11</v>
       </c>
       <c r="G52" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B53" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C53" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="D53" t="s">
         <v>11</v>
       </c>
       <c r="G53" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B54" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C54" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="D54" t="s">
         <v>11</v>
       </c>
       <c r="G54" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B55" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C55" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="D55" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G55" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B56" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C56" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="D56" t="s">
         <v>11</v>
       </c>
       <c r="G56" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B57" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C57" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="D57" t="s">
         <v>11</v>
       </c>
       <c r="G57" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B58" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C58" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="D58" t="s">
         <v>11</v>
       </c>
       <c r="G58" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B59" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C59" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="D59" t="s">
         <v>11</v>
       </c>
       <c r="G59" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B60" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C60" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="D60" t="s">
         <v>11</v>
       </c>
       <c r="G60" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B61" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C61" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="D61" t="s">
         <v>11</v>
       </c>
       <c r="G61" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B62" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C62" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="D62" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G62" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B63" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C63" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="D63" t="s">
         <v>11</v>
       </c>
       <c r="G63" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B64" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C64" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="D64" t="s">
         <v>11</v>
       </c>
       <c r="G64" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B65" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="C65" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="D65" t="s">
         <v>11</v>
       </c>
       <c r="G65" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B66" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C66" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="D66" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G66" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B67" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C67" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="D67" t="s">
         <v>11</v>
       </c>
       <c r="G67" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B68" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C68" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="D68" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G68" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B69" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C69" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="D69" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G69" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B70" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C70" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="D70" t="s">
         <v>11</v>
       </c>
       <c r="G70" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B71" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C71" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="D71" t="s">
         <v>11</v>
       </c>
       <c r="G71" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B72" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C72" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="D72" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G72" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B73" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C73" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="D73" t="s">
         <v>11</v>
       </c>
       <c r="G73" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B74" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C74" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="D74" t="s">
         <v>11</v>
       </c>
       <c r="G74" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B75" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C75" t="s">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="D75" t="s">
         <v>11</v>
       </c>
       <c r="G75" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B76" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C76" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="D76" t="s">
         <v>11</v>
       </c>
       <c r="G76" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B77" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C77" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="D77" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G77" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B78" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C78" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="D78" t="s">
         <v>11</v>
       </c>
       <c r="G78" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B79" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C79" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="D79" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G79" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B80" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="C80" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="D80" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G80" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B81" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C81" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="D81" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G81" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B82" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C82" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="D82" t="s">
         <v>11</v>
       </c>
       <c r="G82" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B83" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C83" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="D83" t="s">
         <v>11</v>
       </c>
       <c r="G83" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B84" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C84" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="D84" t="s">
         <v>11</v>
       </c>
       <c r="G84" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B85" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C85" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="D85" t="s">
         <v>11</v>
       </c>
       <c r="G85" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B86" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C86" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="D86" t="s">
         <v>11</v>
       </c>
       <c r="G86" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B87" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C87" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="D87" t="s">
         <v>11</v>
       </c>
       <c r="G87" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B88" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C88" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="D88" t="s">
         <v>11</v>
       </c>
       <c r="G88" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B89" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C89" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="D89" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G89" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B90" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C90" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="D90" t="s">
         <v>11</v>
       </c>
       <c r="G90" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B91" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C91" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="D91" t="s">
         <v>11</v>
       </c>
       <c r="G91" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B92" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C92" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="D92" t="s">
         <v>11</v>
       </c>
       <c r="G92" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B93" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C93" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="D93" t="s">
         <v>11</v>
       </c>
       <c r="G93" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B94" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C94" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="D94" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G94" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B95" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C95" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="D95" t="s">
         <v>11</v>
       </c>
       <c r="G95" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B96" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C96" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="D96" t="s">
         <v>11</v>
       </c>
       <c r="G96" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B97" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C97" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="D97" t="s">
         <v>11</v>
       </c>
       <c r="G97" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B98" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="C98" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="D98" t="s">
         <v>11</v>
       </c>
       <c r="G98" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B99" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C99" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="D99" t="s">
         <v>11</v>
       </c>
       <c r="G99" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B100" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C100" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="D100" t="s">
         <v>11</v>
       </c>
       <c r="G100" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B101" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C101" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="D101" t="s">
         <v>11</v>
       </c>
       <c r="G101" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B102" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C102" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="D102" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G102" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B103" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C103" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="D103" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G103" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B104" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C104" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="D104" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G104" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B105" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C105" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="D105" t="s">
         <v>11</v>
       </c>
       <c r="G105" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B106" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C106" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="D106" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G106" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B107" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C107" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
       <c r="D107" t="s">
         <v>11</v>
       </c>
       <c r="G107" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B108" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C108" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="D108" t="s">
         <v>11</v>
       </c>
       <c r="G108" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B109" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="C109" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="D109" t="s">
         <v>11</v>
       </c>
       <c r="G109" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B110" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="C110" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="D110" t="s">
         <v>11</v>
       </c>
       <c r="G110" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B111" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C111" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="D111" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G111" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B112" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C112" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="D112" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G112" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B113" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="C113" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="D113" t="s">
         <v>11</v>
       </c>
       <c r="G113" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B114" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C114" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="D114" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G114" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B115" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C115" t="s">
-        <v>130</v>
+        <v>145</v>
       </c>
       <c r="D115" t="s">
         <v>11</v>
       </c>
       <c r="G115" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B116" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C116" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="D116" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G116" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B117" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C117" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="D117" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G117" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B118" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C118" t="s">
-        <v>133</v>
+        <v>148</v>
       </c>
       <c r="D118" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G118" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B119" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C119" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="D119" t="s">
         <v>11</v>
       </c>
       <c r="G119" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B120" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C120" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="D120" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G120" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B121" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C121" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="D121" t="s">
         <v>11</v>
       </c>
       <c r="G121" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B122" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C122" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="D122" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G122" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B123" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C123" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="D123" t="s">
         <v>11</v>
       </c>
       <c r="G123" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B124" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="C124" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="D124" t="s">
         <v>11</v>
       </c>
       <c r="G124" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B125" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="C125" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="D125" t="s">
         <v>11</v>
       </c>
       <c r="G125" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B126" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C126" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="D126" t="s">
         <v>11</v>
       </c>
       <c r="G126" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B127" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C127" t="s">
-        <v>142</v>
+        <v>10</v>
       </c>
       <c r="D127" t="s">
         <v>11</v>
       </c>
       <c r="G127" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B128" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C128" t="s">
-        <v>143</v>
+        <v>12</v>
       </c>
       <c r="D128" t="s">
         <v>11</v>
       </c>
       <c r="G128" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B129" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C129" t="s">
-        <v>144</v>
+        <v>13</v>
       </c>
       <c r="D129" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G129" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B130" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C130" t="s">
-        <v>145</v>
+        <v>14</v>
       </c>
       <c r="D130" t="s">
         <v>11</v>
       </c>
       <c r="G130" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B131" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C131" t="s">
-        <v>146</v>
+        <v>15</v>
       </c>
       <c r="D131" t="s">
         <v>11</v>
       </c>
       <c r="G131" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B132" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C132" t="s">
-        <v>147</v>
+        <v>16</v>
       </c>
       <c r="D132" t="s">
         <v>11</v>
       </c>
       <c r="G132" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B133" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C133" t="s">
-        <v>148</v>
+        <v>17</v>
       </c>
       <c r="D133" t="s">
         <v>11</v>
       </c>
       <c r="G133" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B134" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C134" t="s">
-        <v>149</v>
+        <v>18</v>
       </c>
       <c r="D134" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G134" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B135" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C135" t="s">
-        <v>150</v>
+        <v>19</v>
       </c>
       <c r="D135" t="s">
         <v>11</v>
       </c>
       <c r="G135" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B136" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C136" t="s">
-        <v>151</v>
+        <v>20</v>
       </c>
       <c r="D136" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G136" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B137" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C137" t="s">
-        <v>152</v>
+        <v>21</v>
       </c>
       <c r="D137" t="s">
         <v>11</v>
       </c>
       <c r="G137" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B138" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C138" t="s">
-        <v>153</v>
+        <v>22</v>
       </c>
       <c r="D138" t="s">
         <v>11</v>
       </c>
       <c r="G138" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B139" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="C139" t="s">
-        <v>154</v>
+        <v>23</v>
       </c>
       <c r="D139" t="s">
         <v>11</v>
       </c>
       <c r="G139" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B140" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C140" t="s">
-        <v>155</v>
+        <v>24</v>
       </c>
       <c r="D140" t="s">
         <v>11</v>
       </c>
       <c r="G140" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="B141" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C141" t="s">
-        <v>156</v>
+        <v>25</v>
       </c>
       <c r="D141" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="G141" t="s">
-        <v>12</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>8</v>
+      </c>
+      <c r="B142" t="s">
+        <v>9</v>
+      </c>
+      <c r="C142" t="s">
+        <v>26</v>
+      </c>
+      <c r="D142" t="s">
+        <v>11</v>
+      </c>
+      <c r="G142" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H1" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H142">
+      <sortCondition ref="G1"/>
+    </sortState>
+  </autoFilter>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="E2:E141" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="E2:E142" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>BilledeValgListe</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:G141" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="F2:G142" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"X"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4852,828 +4647,6 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D73"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="45" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="40" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
-        <v>316</v>
-      </c>
-      <c r="C2" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>317</v>
-      </c>
-      <c r="C3" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>318</v>
-      </c>
-      <c r="C4" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>319</v>
-      </c>
-      <c r="C5" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>320</v>
-      </c>
-      <c r="C6" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>321</v>
-      </c>
-      <c r="C7" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" t="s">
-        <v>322</v>
-      </c>
-      <c r="C8" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>323</v>
-      </c>
-      <c r="C9" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>324</v>
-      </c>
-      <c r="C10" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" t="s">
-        <v>325</v>
-      </c>
-      <c r="C11" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" t="s">
-        <v>326</v>
-      </c>
-      <c r="C12" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>8</v>
-      </c>
-      <c r="B13" t="s">
-        <v>327</v>
-      </c>
-      <c r="C13" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>8</v>
-      </c>
-      <c r="B14" t="s">
-        <v>328</v>
-      </c>
-      <c r="C14" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>8</v>
-      </c>
-      <c r="B15" t="s">
-        <v>329</v>
-      </c>
-      <c r="C15" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" t="s">
-        <v>330</v>
-      </c>
-      <c r="C16" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" t="s">
-        <v>331</v>
-      </c>
-      <c r="C17" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>8</v>
-      </c>
-      <c r="B18" t="s">
-        <v>332</v>
-      </c>
-      <c r="C18" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B19" t="s">
-        <v>333</v>
-      </c>
-      <c r="C19" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>8</v>
-      </c>
-      <c r="B20" t="s">
-        <v>334</v>
-      </c>
-      <c r="C20" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>8</v>
-      </c>
-      <c r="B21" t="s">
-        <v>335</v>
-      </c>
-      <c r="C21" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>8</v>
-      </c>
-      <c r="B22" t="s">
-        <v>336</v>
-      </c>
-      <c r="C22" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>8</v>
-      </c>
-      <c r="B23" t="s">
-        <v>337</v>
-      </c>
-      <c r="C23" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>8</v>
-      </c>
-      <c r="B24" t="s">
-        <v>338</v>
-      </c>
-      <c r="C24" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>339</v>
-      </c>
-      <c r="B25" t="s">
-        <v>340</v>
-      </c>
-      <c r="C25" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>339</v>
-      </c>
-      <c r="B26" t="s">
-        <v>341</v>
-      </c>
-      <c r="C26" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>339</v>
-      </c>
-      <c r="B27" t="s">
-        <v>342</v>
-      </c>
-      <c r="C27" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>339</v>
-      </c>
-      <c r="B28" t="s">
-        <v>343</v>
-      </c>
-      <c r="C28" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>339</v>
-      </c>
-      <c r="B29" t="s">
-        <v>344</v>
-      </c>
-      <c r="C29" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>339</v>
-      </c>
-      <c r="B30" t="s">
-        <v>345</v>
-      </c>
-      <c r="C30" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>339</v>
-      </c>
-      <c r="B31" t="s">
-        <v>346</v>
-      </c>
-      <c r="C31" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>339</v>
-      </c>
-      <c r="B32" t="s">
-        <v>347</v>
-      </c>
-      <c r="C32" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>339</v>
-      </c>
-      <c r="B33" t="s">
-        <v>348</v>
-      </c>
-      <c r="C33" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>339</v>
-      </c>
-      <c r="B34" t="s">
-        <v>349</v>
-      </c>
-      <c r="C34" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>339</v>
-      </c>
-      <c r="B35" t="s">
-        <v>350</v>
-      </c>
-      <c r="C35" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>339</v>
-      </c>
-      <c r="B36" t="s">
-        <v>351</v>
-      </c>
-      <c r="C36" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>339</v>
-      </c>
-      <c r="B37" t="s">
-        <v>352</v>
-      </c>
-      <c r="C37" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>339</v>
-      </c>
-      <c r="B38" t="s">
-        <v>353</v>
-      </c>
-      <c r="C38" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>339</v>
-      </c>
-      <c r="B39" t="s">
-        <v>354</v>
-      </c>
-      <c r="C39" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>339</v>
-      </c>
-      <c r="B40" t="s">
-        <v>355</v>
-      </c>
-      <c r="C40" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>339</v>
-      </c>
-      <c r="B41" t="s">
-        <v>356</v>
-      </c>
-      <c r="C41" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>339</v>
-      </c>
-      <c r="B42" t="s">
-        <v>357</v>
-      </c>
-      <c r="C42" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>339</v>
-      </c>
-      <c r="B43" t="s">
-        <v>358</v>
-      </c>
-      <c r="C43" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>339</v>
-      </c>
-      <c r="B44" t="s">
-        <v>359</v>
-      </c>
-      <c r="C44" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>339</v>
-      </c>
-      <c r="B45" t="s">
-        <v>360</v>
-      </c>
-      <c r="C45" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>339</v>
-      </c>
-      <c r="B46" t="s">
-        <v>361</v>
-      </c>
-      <c r="C46" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>339</v>
-      </c>
-      <c r="B47" t="s">
-        <v>362</v>
-      </c>
-      <c r="C47" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>339</v>
-      </c>
-      <c r="B48" t="s">
-        <v>363</v>
-      </c>
-      <c r="C48" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>339</v>
-      </c>
-      <c r="B49" t="s">
-        <v>364</v>
-      </c>
-      <c r="C49" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>339</v>
-      </c>
-      <c r="B50" t="s">
-        <v>366</v>
-      </c>
-      <c r="C50" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>339</v>
-      </c>
-      <c r="B51" t="s">
-        <v>367</v>
-      </c>
-      <c r="C51" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>339</v>
-      </c>
-      <c r="B52" t="s">
-        <v>368</v>
-      </c>
-      <c r="C52" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>339</v>
-      </c>
-      <c r="B53" t="s">
-        <v>369</v>
-      </c>
-      <c r="C53" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>339</v>
-      </c>
-      <c r="B54" t="s">
-        <v>370</v>
-      </c>
-      <c r="C54" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>339</v>
-      </c>
-      <c r="B55" t="s">
-        <v>371</v>
-      </c>
-      <c r="C55" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>339</v>
-      </c>
-      <c r="B56" t="s">
-        <v>372</v>
-      </c>
-      <c r="C56" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>339</v>
-      </c>
-      <c r="B57" t="s">
-        <v>373</v>
-      </c>
-      <c r="C57" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>339</v>
-      </c>
-      <c r="B58" t="s">
-        <v>374</v>
-      </c>
-      <c r="C58" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>339</v>
-      </c>
-      <c r="B59" t="s">
-        <v>375</v>
-      </c>
-      <c r="C59" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>339</v>
-      </c>
-      <c r="B60" t="s">
-        <v>376</v>
-      </c>
-      <c r="C60" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>339</v>
-      </c>
-      <c r="B61" t="s">
-        <v>377</v>
-      </c>
-      <c r="C61" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>339</v>
-      </c>
-      <c r="B62" t="s">
-        <v>378</v>
-      </c>
-      <c r="C62" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>339</v>
-      </c>
-      <c r="B63" t="s">
-        <v>379</v>
-      </c>
-      <c r="C63" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>339</v>
-      </c>
-      <c r="B64" t="s">
-        <v>380</v>
-      </c>
-      <c r="C64" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>339</v>
-      </c>
-      <c r="B65" t="s">
-        <v>381</v>
-      </c>
-      <c r="C65" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>339</v>
-      </c>
-      <c r="B66" t="s">
-        <v>382</v>
-      </c>
-      <c r="C66" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>339</v>
-      </c>
-      <c r="B67" t="s">
-        <v>383</v>
-      </c>
-      <c r="C67" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>339</v>
-      </c>
-      <c r="B68" t="s">
-        <v>384</v>
-      </c>
-      <c r="C68" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>339</v>
-      </c>
-      <c r="B69" t="s">
-        <v>385</v>
-      </c>
-      <c r="C69" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>339</v>
-      </c>
-      <c r="B70" t="s">
-        <v>386</v>
-      </c>
-      <c r="C70" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>339</v>
-      </c>
-      <c r="B71" t="s">
-        <v>387</v>
-      </c>
-      <c r="C71" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>339</v>
-      </c>
-      <c r="B72" t="s">
-        <v>388</v>
-      </c>
-      <c r="C72" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>339</v>
-      </c>
-      <c r="B73" t="s">
-        <v>389</v>
-      </c>
-      <c r="C73" t="s">
-        <v>250</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5683,7 +4656,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>390</v>
+        <v>315</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -5691,50 +4664,50 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>391</v>
+        <v>316</v>
       </c>
       <c r="B3" t="s">
-        <v>392</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>393</v>
+        <v>318</v>
       </c>
       <c r="B4" t="s">
-        <v>394</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>395</v>
+        <v>320</v>
       </c>
       <c r="B5" t="s">
-        <v>396</v>
+        <v>321</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>397</v>
+        <v>322</v>
       </c>
       <c r="B6" t="s">
-        <v>398</v>
+        <v>323</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>399</v>
+        <v>324</v>
       </c>
       <c r="B7" t="s">
-        <v>400</v>
+        <v>325</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>401</v>
+        <v>326</v>
       </c>
       <c r="B8" t="s">
-        <v>402</v>
+        <v>327</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -5742,42 +4715,42 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>403</v>
+        <v>328</v>
       </c>
       <c r="B10" t="s">
-        <v>404</v>
+        <v>329</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>403</v>
+        <v>328</v>
       </c>
       <c r="B11" t="s">
-        <v>405</v>
+        <v>330</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>403</v>
+        <v>328</v>
       </c>
       <c r="B12" t="s">
-        <v>406</v>
+        <v>331</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>403</v>
+        <v>328</v>
       </c>
       <c r="B13" t="s">
-        <v>407</v>
+        <v>332</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>403</v>
+        <v>328</v>
       </c>
       <c r="B14" t="s">
-        <v>408</v>
+        <v>333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gem mine valg (sport + danske backdrops) 2026-10-06 21:36:20
</commit_message>
<xml_diff>
--- a/data/sport_artwork_review.xlsx
+++ b/data/sport_artwork_review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EPGoal\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC18EA0-DCB6-45EF-93CD-F60137BD7D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF09C96-1A5E-4FAB-B85C-2E6A7D06C6D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="337">
   <si>
     <t>Kanalgruppe</t>
   </si>
@@ -1034,6 +1034,9 @@
   </si>
   <si>
     <t>Rækker der ikke længere er aktuelle, men SOM havde et udfyldt valg (og ikke er ignoreret), havner i arket 'Forsvundne (havde valg)' - intet forsvinder usporligt.</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -1398,7 +1401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H143"/>
+  <dimension ref="A1:H144"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -3845,6 +3848,14 @@
       </c>
       <c r="D143" t="s">
         <v>11</v>
+      </c>
+      <c r="G143" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G144" t="s">
+        <v>336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-opdater EPGOAL 2026-10-09 15:25:44
</commit_message>
<xml_diff>
--- a/data/sport_artwork_review.xlsx
+++ b/data/sport_artwork_review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EPGoal\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_A948C11FF65F11CE9343156F17823D11BF5071D9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_A948C11FF62F17DBF77301677BC03411BF507E45" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2409" uniqueCount="757">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2434" uniqueCount="757">
   <si>
     <t>Kanalgruppe</t>
   </si>
@@ -3418,6 +3418,9 @@
       <c r="D52" t="s">
         <v>98</v>
       </c>
+      <c r="G52" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
@@ -3617,6 +3620,9 @@
       <c r="D66" t="s">
         <v>30</v>
       </c>
+      <c r="G66" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
@@ -3774,6 +3780,9 @@
       <c r="D77" t="s">
         <v>30</v>
       </c>
+      <c r="G77" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
@@ -4050,7 +4059,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>8</v>
       </c>
@@ -4064,7 +4073,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>8</v>
       </c>
@@ -4078,7 +4087,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>8</v>
       </c>
@@ -4092,7 +4101,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>8</v>
       </c>
@@ -4106,7 +4115,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>8</v>
       </c>
@@ -4120,7 +4129,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>8</v>
       </c>
@@ -4134,7 +4143,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>8</v>
       </c>
@@ -4147,8 +4156,11 @@
       <c r="D103" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G103" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>8</v>
       </c>
@@ -4161,8 +4173,11 @@
       <c r="D104" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G104" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>8</v>
       </c>
@@ -4176,7 +4191,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>8</v>
       </c>
@@ -4190,7 +4205,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>8</v>
       </c>
@@ -4203,8 +4218,11 @@
       <c r="D107" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G107" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>8</v>
       </c>
@@ -4218,7 +4236,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>8</v>
       </c>
@@ -4232,7 +4250,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>8</v>
       </c>
@@ -4246,7 +4264,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>8</v>
       </c>
@@ -4260,7 +4278,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>8</v>
       </c>
@@ -4301,6 +4319,9 @@
       <c r="D114" t="s">
         <v>30</v>
       </c>
+      <c r="G114" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
@@ -4315,6 +4336,9 @@
       <c r="D115" t="s">
         <v>30</v>
       </c>
+      <c r="G115" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
@@ -4329,6 +4353,9 @@
       <c r="D116" t="s">
         <v>30</v>
       </c>
+      <c r="G116" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
@@ -4530,6 +4557,9 @@
       </c>
       <c r="D130" t="s">
         <v>30</v>
+      </c>
+      <c r="G130" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.25">
@@ -5061,6 +5091,9 @@
       <c r="D167" t="s">
         <v>30</v>
       </c>
+      <c r="G167" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
@@ -5103,6 +5136,9 @@
       <c r="D170" t="s">
         <v>30</v>
       </c>
+      <c r="G170" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
@@ -5131,6 +5167,9 @@
       <c r="D172" t="s">
         <v>30</v>
       </c>
+      <c r="G172" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
@@ -5159,6 +5198,9 @@
       <c r="D174" t="s">
         <v>30</v>
       </c>
+      <c r="G174" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
@@ -5188,7 +5230,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>243</v>
       </c>
@@ -5201,8 +5243,11 @@
       <c r="D177" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G177" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>243</v>
       </c>
@@ -5216,7 +5261,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>243</v>
       </c>
@@ -5230,7 +5275,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>243</v>
       </c>
@@ -5244,7 +5289,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>243</v>
       </c>
@@ -5258,7 +5303,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>243</v>
       </c>
@@ -5272,7 +5317,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>243</v>
       </c>
@@ -5286,7 +5331,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>243</v>
       </c>
@@ -5300,7 +5345,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>243</v>
       </c>
@@ -5314,7 +5359,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>243</v>
       </c>
@@ -5328,7 +5373,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>243</v>
       </c>
@@ -5342,7 +5387,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>243</v>
       </c>
@@ -5356,7 +5401,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>243</v>
       </c>
@@ -5370,7 +5415,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>243</v>
       </c>
@@ -5384,7 +5429,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>243</v>
       </c>
@@ -5398,7 +5443,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>243</v>
       </c>
@@ -5412,7 +5457,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>243</v>
       </c>
@@ -5426,7 +5471,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>243</v>
       </c>
@@ -5440,7 +5485,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>243</v>
       </c>
@@ -5454,7 +5499,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>243</v>
       </c>
@@ -5468,7 +5513,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>243</v>
       </c>
@@ -5482,7 +5527,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>243</v>
       </c>
@@ -5496,7 +5541,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>243</v>
       </c>
@@ -5509,8 +5554,11 @@
       <c r="D199" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G199" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>243</v>
       </c>
@@ -5523,8 +5571,11 @@
       <c r="D200" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G200" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>243</v>
       </c>
@@ -5538,7 +5589,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>243</v>
       </c>
@@ -5552,7 +5603,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>243</v>
       </c>
@@ -5566,7 +5617,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>243</v>
       </c>
@@ -5580,7 +5631,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>243</v>
       </c>
@@ -5594,7 +5645,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>243</v>
       </c>
@@ -5608,7 +5659,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>243</v>
       </c>
@@ -5622,7 +5673,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>243</v>
       </c>
@@ -5635,8 +5686,11 @@
       <c r="D208" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G208" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>243</v>
       </c>
@@ -5650,7 +5704,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>243</v>
       </c>
@@ -5664,7 +5718,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>243</v>
       </c>
@@ -5677,8 +5731,11 @@
       <c r="D211" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G211" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>243</v>
       </c>
@@ -5692,7 +5749,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>243</v>
       </c>
@@ -5706,7 +5763,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>243</v>
       </c>
@@ -5720,7 +5777,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>243</v>
       </c>
@@ -5734,7 +5791,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>243</v>
       </c>
@@ -5748,7 +5805,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>243</v>
       </c>
@@ -5762,7 +5819,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>243</v>
       </c>
@@ -5776,7 +5833,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>243</v>
       </c>
@@ -5790,7 +5847,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>243</v>
       </c>
@@ -5804,7 +5861,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>243</v>
       </c>
@@ -5818,7 +5875,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>243</v>
       </c>
@@ -5832,7 +5889,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>243</v>
       </c>
@@ -5845,8 +5902,11 @@
       <c r="D223" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G223" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>243</v>
       </c>
@@ -5860,7 +5920,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>243</v>
       </c>
@@ -5874,7 +5934,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>243</v>
       </c>
@@ -5888,7 +5948,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>243</v>
       </c>
@@ -5901,8 +5961,11 @@
       <c r="D227" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G227" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>243</v>
       </c>
@@ -5916,7 +5979,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>243</v>
       </c>
@@ -5930,7 +5993,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>243</v>
       </c>
@@ -5944,7 +6007,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>243</v>
       </c>
@@ -5957,8 +6020,11 @@
       <c r="D231" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="232" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G231" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>243</v>
       </c>
@@ -5972,7 +6038,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>243</v>
       </c>
@@ -5986,7 +6052,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>243</v>
       </c>
@@ -5999,8 +6065,11 @@
       <c r="D234" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G234" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>243</v>
       </c>
@@ -6013,8 +6082,11 @@
       <c r="D235" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G235" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>243</v>
       </c>
@@ -6027,8 +6099,11 @@
       <c r="D236" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="G236" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>243</v>
       </c>
@@ -6042,7 +6117,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="238" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>243</v>
       </c>
@@ -6056,7 +6131,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="239" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>243</v>
       </c>
@@ -6070,7 +6145,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="240" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>243</v>
       </c>

</xml_diff>